<commit_message>
Ajout de backlog.xlsx aux fichiers référencés pour cohérence dans le pack généré
</commit_message>
<xml_diff>
--- a/cahier des charges/backlog.xlsx
+++ b/cahier des charges/backlog.xlsx
@@ -59,9 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -505,6 +508,11 @@
           <t>Besoins testables</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Point d'effort prestataire (1er niveau)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -566,6 +574,10 @@
 Étant donné un fichier non conforme (extension non supportée, colonnes obligatoires manquantes), Quand l'administrateur tente l'import, Alors l'import est refusée et un message d'erreur explicite liste les anomalies détectées.</t>
         </is>
       </c>
+      <c r="M2">
+        <f>SUMIF('Besoins testables'!$D:$D,$A2,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -618,6 +630,7 @@
           <t>En tant qu'administrateur expert data, je veux connecter une API externe afin d'alimenter la plateforme sans fichier.</t>
         </is>
       </c>
+      <c r="M3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -680,6 +693,10 @@
           <t>Étant donné une source de données fichier, Quand l'administrateur définit une planification (fréquence journalière, hebdomadaire, mensuelle, heure d'exécution), Alors l'import est exécuté automatiquement à l'échéance prévue, Et chaque exécution est tracée (date, heure, source, résultat, volumétrie). - Quand un import planifié échoue, Alors son statut passe à « échec », l'événement est journalisé avec le motif, Et les exécutions suivantes restent programmées. - Quand la planification est modifiée ou supprimée, Alors seules les nouvelles exécutions respectent la configuration courante, les exécutions déjà tracées restant inchangées. - Quand deux imports planifiés se chevauchent, Alors le système les sérialise ou refuse le chevauchement sans perte de données.
 Étant donné un import planifié sans fichier source disponible à l'échéance, Alors l'exécution est signalée en échec avec un motif explicite, Et aucune donnée partielle ou vide n'est enregistrée.</t>
         </is>
+      </c>
+      <c r="M4">
+        <f>SUMIF('Besoins testables'!$D:$D,$A4,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -745,6 +762,10 @@
 Étant donné une valeur numérique hors plage ou un format inattendu, Quand la normalisation échoue pour cette ligne, Alors la ligne est marquée « non normalisée », Et le reste du jeu est traité sans blocage global. - Quand aucune règle de normalisation n'existe pour une colonne obligatoire, Alors l'import est refusée avec un message renvoyant vers la configuration de la source. - Quand un jeu de données normalisé est réimporté, Alors les mêmes règles produisent les mêmes valeurs (reproductibilité de la normalisation).</t>
         </is>
       </c>
+      <c r="M5">
+        <f>SUMIF('Besoins testables'!$D:$D,$A5,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -809,6 +830,10 @@
 Étant donné un fichier corrigé après un rejet, Quand l'administrateur relance l'import, Alors seules les nouvelles anomalies sont signalées, les lignes précédemment corrigées n'apparaissant plus dans le rapport.</t>
         </is>
       </c>
+      <c r="M6">
+        <f>SUMIF('Besoins testables'!$D:$D,$A6,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -872,6 +897,10 @@
 Étant donné une date de référence, Quand l'administrateur interroge l'historique, Alors il peut reconstituer l'état du jeu de données tel qu'il existait à cette date. - Quand une nouvelle version est enregistrée, Alors son horodatage, sa source et le traitement d'origine sont tracés. - Quand une opération de réécriture est demandée, Alors aucune donnée existante n'est écrasée sans création préalable d'une nouvelle version (aucune suppression destructive). ### EPIC 1bis — Catalogage des données</t>
         </is>
       </c>
+      <c r="M7">
+        <f>SUMIF('Besoins testables'!$D:$D,$A7,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -924,6 +953,7 @@
           <t>En tant qu'administrateur expert data, je veux rejouer un traitement afin de recalculer un jeu de données après correction.</t>
         </is>
       </c>
+      <c r="M8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -988,6 +1018,10 @@
 Étant donné un jeu de données non encore intégré, Quand l'administrateur tente de l'enregistrer, Alors l'enregistrement est refusée : le catalogue ne référence que des données réellement disponibles dans la plateforme.</t>
         </is>
       </c>
+      <c r="M9">
+        <f>SUMIF('Besoins testables'!$D:$D,$A9,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1052,6 +1086,10 @@
 Étant donné une licence non autorisée ou une date de mise à jour future, Quand l'enregistrement est tenté, Alors il est refusé avec un message d'erreur explicite.</t>
         </is>
       </c>
+      <c r="M10">
+        <f>SUMIF('Besoins testables'!$D:$D,$A10,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1109,6 +1147,7 @@
           <t>En tant qu'administrateur expert data, je veux modifier les métadonnées afin de maintenir le catalogue à jour.</t>
         </is>
       </c>
+      <c r="M11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1168,6 +1207,10 @@
 Étant donné un jeu de données sans licence renseignée, Quand sa fiche est consultée, Alors la mention « licence non renseignée » est affichée (aucune valeur par défaut trompeuse). - Quand la fiche est consultée depuis le catalogue, Alors l'utilisateur voit les métadonnées de qualité associées (EPIC 2) si elles existent.</t>
         </is>
       </c>
+      <c r="M12">
+        <f>SUMIF('Besoins testables'!$D:$D,$A12,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1220,6 +1263,7 @@
           <t>En tant qu'administrateur expert data, je veux rechercher un jeu de données afin de le retrouver rapidement dans le catalogue.</t>
         </is>
       </c>
+      <c r="M13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1272,6 +1316,7 @@
           <t>En tant qu'administrateur expert data, je veux filtrer les jeux de données selon des critères afin de restreindre la liste du catalogue.</t>
         </is>
       </c>
+      <c r="M14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1331,6 +1376,10 @@
 Étant donné un indicateur sans dépendance déclarée, Quand la page est ouverte, Alors un message indique l'absence de relations tracées plutôt qu'un graphe vide. - Quand l'indicateur est recalculé sur de nouvelles données, Alors le graphe reflète les relations de la version de calcul la plus récente.</t>
         </is>
       </c>
+      <c r="M15">
+        <f>SUMIF('Besoins testables'!$D:$D,$A15,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1383,6 +1432,7 @@
           <t>En tant qu'administrateur expert data, je veux tracer les transformations appliquées à un jeu de données afin d'en garantir la reproductibilité.</t>
         </is>
       </c>
+      <c r="M16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1435,6 +1485,7 @@
           <t>En tant qu'administrateur expert data, je veux identifier une donnée comme source ou dérivée afin de clarifier sa place dans la chaîne.</t>
         </is>
       </c>
+      <c r="M17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1500,6 +1551,10 @@
 Étant donné un import sans identifiant de jeu identifiable, Quand l'alimentation du catalogue est tentée, Alors l'import est signalé en échec partiel avec le motif.</t>
         </is>
       </c>
+      <c r="M18">
+        <f>SUMIF('Besoins testables'!$D:$D,$A18,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1557,6 +1612,7 @@
           <t>En tant qu'administrateur expert data, je veux relier un jeu de données à un traitement afin d'en retracer l'élaboration.</t>
         </is>
       </c>
+      <c r="M19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1621,6 +1677,10 @@
 Étant donné un indicateur non défini dans le référentiel, Quand l'administrateur tente de l'enregistrer, Alors l'enregistrement est refusé avec un message renvoyant vers la définition de l'indicateur (US3.5). - Quand un indicateur dérivé est recalculé, Alors la version cataloguée est mise à jour, Et la traçabilité du calcul (date, version de la méthode, données utilisées) est conservée. ### EPIC 2 — Qualité des données</t>
         </is>
       </c>
+      <c r="M20">
+        <f>SUMIF('Besoins testables'!$D:$D,$A20,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1673,6 +1733,7 @@
           <t>En tant qu'administrateur expert data, je veux consulter les métadonnées d'un indicateur afin d'en vérifier la définition et la méthode.</t>
         </is>
       </c>
+      <c r="M21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1725,6 +1786,7 @@
           <t>En tant qu'administrateur expert data, je veux ajouter un nouveau jeu de données sans modifier la structure afin d'étendre le catalogue à moindre coût.</t>
         </is>
       </c>
+      <c r="M22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1777,6 +1839,7 @@
           <t>En tant qu'administrateur expert data, je veux historiser les modifications des métadonnées afin de tracer les évolutions du catalogue.</t>
         </is>
       </c>
+      <c r="M23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1837,6 +1900,10 @@
 Étant donné un jeu sans règles de détection configurées, Quand le contrôle est exécuté, Alors aucune valeur aberrante n'est signalée et le jeu est qualifié « non contrôlé ».</t>
         </is>
       </c>
+      <c r="M24">
+        <f>SUMIF('Besoins testables'!$D:$D,$A24,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1889,6 +1956,7 @@
           <t>En tant qu'administrateur expert data, je veux vérifier la cohérence temporelle afin de détecter les incohérences de dates.</t>
         </is>
       </c>
+      <c r="M25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1941,6 +2009,7 @@
           <t>En tant qu'administrateur expert data, je veux vérifier la cohérence spatiale afin de détecter les incohérences géographiques.</t>
         </is>
       </c>
+      <c r="M26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1998,6 +2067,10 @@
           <t>Étant donné un jeu de données avec des champs obligatoires définis, Quand le taux de complétude est calculé, Alors il correspond au pourcentage de valeurs renseignées sur les valeurs attendues, par champ et par jeu, Et le résultat est stocké comme métadonnée de qualité. - Quand un taux est calculé, Alors la période et la version du jeu de données utilisées pour le calcul sont précisées.
 Étant donné un seuil de complétude configuré (par défaut 95 %), Quand le taux calculé est inférieur au seuil, Alors le jeu est marqué comme sous le seuil, Et l'information est reportée sur sa fiche qualité. - Quand un jeu est mis à jour (nouvel import, corrections), Alors le taux est recalculé sur la dernière version, sans perte des taux historiques. - Quand le taux de complétude d'un jeu sert au calcul d'un indicateur (EPIC 4), Alors il est exploitable de façon automatisée (filtrage ou marquage du résultat).</t>
         </is>
+      </c>
+      <c r="M27">
+        <f>SUMIF('Besoins testables'!$D:$D,$A27,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -2058,6 +2131,10 @@
 Étant donné un jeu sans métadonnées de qualité renseignées, Quand l'évaluation est demandée, Alors aucune classe n'est attribuée : le jeu est qualifié « fiabilité non évaluée » (pas de note par défaut trompeuse). - Quand une classe de fiabilité est disponible, Alors elle est exploitable par les traitements ultérieurs (filtrage, affichage différencié).</t>
         </is>
       </c>
+      <c r="M28">
+        <f>SUMIF('Besoins testables'!$D:$D,$A28,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2117,6 +2194,10 @@
 Étant donné un jeu de données non intégré dans la plateforme, Quand l'administrateur tente d'ajouter des métadonnées de qualité, Alors l'opération est refusée avec un message explicite. - Quand l'administrateur consulte la fiche qualité, Alors il voit un résumé : date du dernier contrôle, classe de fiabilité, taux de complétude, nombre d'anomalies ouvertes. ### EPIC 3 — Référentiels</t>
         </is>
       </c>
+      <c r="M29">
+        <f>SUMIF('Besoins testables'!$D:$D,$A29,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2169,6 +2250,7 @@
           <t>En tant qu'administrateur expert data, je veux visualiser la qualité afin de repérer les jeux de données fiables.</t>
         </is>
       </c>
+      <c r="M30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2228,6 +2310,10 @@
 Étant donné un BVAEP auquel des données ou des captages sont rattachés, Quand l'administrateur tente de le supprimer, Alors la suppression est refusée tant qu'aucun réaffectement explicite n'a été effectué.</t>
         </is>
       </c>
+      <c r="M31">
+        <f>SUMIF('Besoins testables'!$D:$D,$A31,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2286,6 +2372,10 @@
 Étant donné un identifiant de captage déjà utilisé, Quand la création est tentée, Alors elle est refusée avec un message explicite.</t>
         </is>
       </c>
+      <c r="M32">
+        <f>SUMIF('Besoins testables'!$D:$D,$A32,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2338,6 +2428,7 @@
           <t>En tant qu'administrateur expert data, je veux gérer les périmètres de protection afin de les représenter sur la carte.</t>
         </is>
       </c>
+      <c r="M33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2398,6 +2489,10 @@
 Étant donné une résolution non supportée, Quand l'administrateur tente de la configurer, Alors l'opération est refusée avec la liste des résolutions disponibles.</t>
         </is>
       </c>
+      <c r="M34">
+        <f>SUMIF('Besoins testables'!$D:$D,$A34,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2457,6 +2552,10 @@
 Étant donné un indicateur déjà défini sous le même nom ou le même identifiant, Quand la définition est tentée, Alors elle est refusée avec un message explicite. ### EPIC 4 — Calcul d'indicateurs</t>
         </is>
       </c>
+      <c r="M35">
+        <f>SUMIF('Besoins testables'!$D:$D,$A35,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2509,6 +2608,7 @@
           <t>En tant qu'administrateur plateforme, je veux gérer les profils utilisateurs et leurs droits afin de contrôler les accès à la plateforme.</t>
         </is>
       </c>
+      <c r="M36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2561,6 +2661,7 @@
           <t>En tant qu'administrateur expert data, je veux versionner les référentiels afin de conserver l'historique de leurs évolutions.</t>
         </is>
       </c>
+      <c r="M37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2626,6 +2727,10 @@
 Étant donné un indicateur sans méthode complète ou sans données sources, Quand le calcul est demandé, Alors il est refusé avec un message explicite.</t>
         </is>
       </c>
+      <c r="M38">
+        <f>SUMIF('Besoins testables'!$D:$D,$A38,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2691,6 +2796,10 @@
 Étant donné un indicateur sans règle d'agrégation spatiale définie, Quand l'agrégation à l'échelle BV est demandée, Alors elle est refusée avec un message explicite.</t>
         </is>
       </c>
+      <c r="M39">
+        <f>SUMIF('Besoins testables'!$D:$D,$A39,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2755,6 +2864,10 @@
 Étant donné une période demandée dépassant l'historique disponible, Quand l'agrégation est exécutée, Alors elle est limitée à l'historique existant et l'écart est signalé, ou refusée si aucune donnée ne couvre la période. - Quand un indicateur est produit à plusieurs granularités temporelles, Alors le périmètre de calcul (données incluses, période couverte) est documenté pour garantir la comparabilité des séries.</t>
         </is>
       </c>
+      <c r="M40">
+        <f>SUMIF('Besoins testables'!$D:$D,$A40,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2807,6 +2920,7 @@
           <t>En tant qu'administrateur expert data, je veux paramétrer un calcul afin d'ajuster les règles de production de l'indicateur.</t>
         </is>
       </c>
+      <c r="M41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2865,6 +2979,10 @@
 Étant donné une combinaison de filtres ne sélectionnant aucune donnée, Quand le calcul est demandé, Alors il est refusé avec le message « aucun jeu de données ne correspond aux filtres appliqués ». - Quand l'administrateur consulte la configuration du calcul, Alors il voit un résumé des critères retenus (période, sources, territoires, seuil de qualité) avant exécution.</t>
         </is>
       </c>
+      <c r="M42">
+        <f>SUMIF('Besoins testables'!$D:$D,$A42,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2917,6 +3035,7 @@
           <t>En tant qu'administrateur expert data, je veux versionner un indicateur afin de conserver la traçabilité de ses évolutions.</t>
         </is>
       </c>
+      <c r="M43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2974,6 +3093,7 @@
           <t>En tant qu'administrateur expert data, je veux recalculer un indicateur afin de mettre à jour les valeurs après correction.</t>
         </is>
       </c>
+      <c r="M44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3031,6 +3151,7 @@
           <t>En tant qu'administrateur expert data, je veux construire un indice composite afin de fournir une base transparente pour l'aide à la décision.</t>
         </is>
       </c>
+      <c r="M45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3088,6 +3209,7 @@
           <t>En tant qu'expert métier eau potable, je veux définir les pondérations de l'analyse multicritère afin d'évaluer le risque réel de dégradation de la ressource.</t>
         </is>
       </c>
+      <c r="M46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3145,6 +3267,7 @@
           <t>En tant qu'expert métier eau potable, je veux tester des scénarios de pondération afin d'analyser l'impact des différents facteurs sur le classement de criticité.</t>
         </is>
       </c>
+      <c r="M47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3202,6 +3325,7 @@
           <t>En tant qu'expert métier eau potable, je veux comparer les scénarios de l'analyse multicritère afin d'identifier la pondération la plus représentative du terrain.</t>
         </is>
       </c>
+      <c r="M48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3259,6 +3383,7 @@
           <t>En tant qu'expert métier eau potable, je veux visualiser la contribution de chaque indicateur au score de criticité afin de comprendre les facteurs de risque dominants.</t>
         </is>
       </c>
+      <c r="M49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3311,6 +3436,7 @@
           <t>En tant qu'administrateur expert data, je veux documenter les méthodes de calcul afin d'assurer la transparence de l'aide à la décision.</t>
         </is>
       </c>
+      <c r="M50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3371,6 +3497,10 @@
 Étant donné une zone sans donnée dans l'emprise, quand la carte est rendue, alors le périmètre reste lisible avec un libellé explicite (pas de fond vide ambigu).</t>
         </is>
       </c>
+      <c r="M51">
+        <f>SUMIF('Besoins testables'!$D:$D,$A51,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3436,6 +3566,10 @@
 Étant donné un changement d'indicateur (via Famille → Thème → Groupe), quand je bascule, alors la légende et les couleurs correspondent immédiatement au nouvel indicateur en conservant la sélection courante.</t>
         </is>
       </c>
+      <c r="M52">
+        <f>SUMIF('Besoins testables'!$D:$D,$A52,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3496,6 +3630,10 @@
 Étant donné un changement d'échelle, quand les unités deviennent trop nombreuses à l'écran, alors la carte propose un regroupement lisible (agrégation visuelle) sans perte de données.</t>
         </is>
       </c>
+      <c r="M53">
+        <f>SUMIF('Besoins testables'!$D:$D,$A53,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3561,6 +3699,10 @@
 Étant donné un point de la série, quand je le survole, alors une infobulle affiche la date et la valeur de l'indicateur.</t>
         </is>
       </c>
+      <c r="M54">
+        <f>SUMIF('Besoins testables'!$D:$D,$A54,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3613,6 +3755,7 @@
           <t>En tant que décideur métier, je veux comparer des territoires afin d'arbitrer les investissements.</t>
         </is>
       </c>
+      <c r="M55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3665,6 +3808,7 @@
           <t>En tant que décideur métier, je veux disposer d'un tableau de bord avancé afin d'avoir une vue agrégée de l'information.</t>
         </is>
       </c>
+      <c r="M56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3725,6 +3869,10 @@
 Étant donné une donnée source mise à jour, quand la fiche est consultée, alors elle reflète la dernière version sans action manuelle.</t>
         </is>
       </c>
+      <c r="M57">
+        <f>SUMIF('Besoins testables'!$D:$D,$A57,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3790,6 +3938,10 @@
 Étant donné le compteur d'unités, quand je bascule d'échelle, alors il reflète immédiatement le nombre d'unités sélectionnées à la nouvelle échelle.</t>
         </is>
       </c>
+      <c r="M58">
+        <f>SUMIF('Besoins testables'!$D:$D,$A58,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3850,6 +4002,10 @@
 Étant donné la carte, les listes et le compteur, quand une sélection est modifiée, alors ils restent cohérents entre eux.</t>
         </is>
       </c>
+      <c r="M59">
+        <f>SUMIF('Besoins testables'!$D:$D,$A59,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3910,6 +4066,10 @@
 Étant donné une recherche sans résultat, quand elle est exécutée, alors un message « Aucun résultat » est affiché, sans rechargement ni erreur.</t>
         </is>
       </c>
+      <c r="M60">
+        <f>SUMIF('Besoins testables'!$D:$D,$A60,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3970,6 +4130,10 @@
 Étant donné l'état courant des facettes, quand je quitte puis reviens sur la vue, alors l'état est restauré ou clairement signalé comme non conservé.</t>
         </is>
       </c>
+      <c r="M61">
+        <f>SUMIF('Besoins testables'!$D:$D,$A61,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4029,6 +4193,10 @@
 Étant donné une puce active, quand je clique sur sa croix de désélection, alors le filtre est retiré et toutes les vues (carte, liste, graphiques) se mettent à jour.
 Étant donné l'ensemble des puces, quand je les retire une à une, alors la sélection initiale est progressivement restituée jusqu'au retour à l'état de départ.</t>
         </is>
+      </c>
+      <c r="M62">
+        <f>SUMIF('Besoins testables'!$D:$D,$A62,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -4091,6 +4259,10 @@
 Étant donné une unité non classable par la règle du preset, quand elle n'est pas retenue, alors elle n'est pas exclue silencieusement et reste consultable.</t>
         </is>
       </c>
+      <c r="M63">
+        <f>SUMIF('Besoins testables'!$D:$D,$A63,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4149,6 +4321,10 @@
 Étant donné une facette décochée, quand je la décoche à nouveau, alors rien ne change (comportement idempotent, sans erreur).
 Étant donné un filtre retiré par décochage, quand je le ré-applique, alors le résultat correspond au résultat initial (pas de dérive de l'état).</t>
         </is>
+      </c>
+      <c r="M64">
+        <f>SUMIF('Besoins testables'!$D:$D,$A64,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -4210,6 +4386,10 @@
 Étant donné une unité retirée, quand un graphique est affiché, alors l'unité n'apparaît plus dans les séries renvoyées.</t>
         </is>
       </c>
+      <c r="M65">
+        <f>SUMIF('Besoins testables'!$D:$D,$A65,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4268,6 +4448,10 @@
 Étant donné une sélection de captages, quand j'ajoute une sélection de BVAEP, alors les deux coexistent et restent affichées distinctement dans les composants dédiés.
 Étant donné la bascule d'échelle, quand je reviens aux captages, alors la sélection de captages d'origine est restituée à l'identique.</t>
         </is>
+      </c>
+      <c r="M66">
+        <f>SUMIF('Besoins testables'!$D:$D,$A66,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -4328,6 +4512,10 @@
 Étant donné un tri en cours, quand je change de mode, alors l'autre mode s'applique immédiatement.
 Étant donné un tri appliqué, quand j'ajoute ou je retire des unités, alors l'ordre est recalculé en conservant le mode choisi.</t>
         </is>
+      </c>
+      <c r="M67">
+        <f>SUMIF('Besoins testables'!$D:$D,$A67,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -4395,6 +4583,10 @@
 Étant donné un calcul exécuté, quand le seuil ou le référentiel ont été modifiés, alors le recalcul est rejouable et trace les paramètres utilisés (seuil, version du référentiel), sans saisie manuelle.</t>
         </is>
       </c>
+      <c r="M68">
+        <f>SUMIF('Besoins testables'!$D:$D,$A68,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4460,6 +4652,10 @@
 Étant donné un référentiel mis à jour (US3.1 / US3.2), quand la carte est rafraîchie, alors le croisement restitué utilise les relations à jour.</t>
         </is>
       </c>
+      <c r="M69">
+        <f>SUMIF('Besoins testables'!$D:$D,$A69,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4520,6 +4716,10 @@
 Étant donné le choix du fond, quand ma préférence est mémorisée, alors elle est ré-appliquée lors des prochaines sessions.</t>
         </is>
       </c>
+      <c r="M70">
+        <f>SUMIF('Besoins testables'!$D:$D,$A70,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4580,6 +4780,10 @@
 Étant donné plusieurs couches actives, quand elles se superposent, alors l'ordre de rendu est stable et la lisibilité est conservée.</t>
         </is>
       </c>
+      <c r="M71">
+        <f>SUMIF('Besoins testables'!$D:$D,$A71,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4640,6 +4844,10 @@
 Étant donné l'indicateur choisi, quand je le valide, alors le catalogue indicateurs et la carte se mettent à jour.</t>
         </is>
       </c>
+      <c r="M72">
+        <f>SUMIF('Besoins testables'!$D:$D,$A72,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4699,6 +4907,10 @@
 Étant donné la règle d'accès, quand je tente d'ouvrir les métadonnées depuis un graphique, alors l'entrée n'est pas activée (accès uniquement depuis la vignette).
 Étant donné une fiche métadonnées d'indicateur, quand elle est consultée, alors elle est cohérente avec le catalogue de référence même si l'indicateur n'est pas encore calculé.</t>
         </is>
+      </c>
+      <c r="M73">
+        <f>SUMIF('Besoins testables'!$D:$D,$A73,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="74">
@@ -4761,6 +4973,10 @@
 Étant donné un indicateur, quand la vue « Carte » (maille H3) est affichée, alors elle est cohérente avec la carte principale (classes et palettes identiques).</t>
         </is>
       </c>
+      <c r="M74">
+        <f>SUMIF('Besoins testables'!$D:$D,$A74,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4821,6 +5037,10 @@
 Étant donné les droits du profil, quand un indicateur n'est pas autorisé, alors il est absent de la liste pour ce profil, sans message d'erreur.</t>
         </is>
       </c>
+      <c r="M75">
+        <f>SUMIF('Besoins testables'!$D:$D,$A75,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4880,6 +5100,10 @@
 Étant donné une pré-sélection appliquée, quand le volet droit est rendu, alors l'indicateur proposé est en cohérence avec les thèmes et le groupe sélectionnés.
 Étant donné une navigation entre familles, quand je change de tab, alors la pré-sélection de la nouvelle famille s'applique sans confusion avec la précédente. --- EPIC 7 — Aide à la décision</t>
         </is>
+      </c>
+      <c r="M76">
+        <f>SUMIF('Besoins testables'!$D:$D,$A76,'Besoins testables'!$O:$O)</f>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -4942,6 +5166,10 @@
 Étant donné un volume important, quand l'export est demandé, alors le résultat est complet (pagination interne, sans perte silencieuse) et la préparation est signalée si nécessaire.</t>
         </is>
       </c>
+      <c r="M77">
+        <f>SUMIF('Besoins testables'!$D:$D,$A77,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4994,6 +5222,7 @@
           <t>En tant qu'administrateur expert data, je veux exporter au format SIG afin de réutiliser les données dans un logiciel cartographique.</t>
         </is>
       </c>
+      <c r="M78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5051,6 +5280,7 @@
           <t>En tant que décideur métier, je veux générer un rapport PDF afin de présenter les résultats au conseil municipal et formaliser la prise de décision.</t>
         </is>
       </c>
+      <c r="M79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5103,6 +5333,7 @@
           <t>En tant qu'administrateur expert data, je veux partager un lien afin de transmettre une vue des données à un collaborateur.</t>
         </is>
       </c>
+      <c r="M80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5155,6 +5386,7 @@
           <t>En tant qu'administrateur expert data, je veux accéder aux données via une API afin de les réutiliser dans d'autres systèmes.</t>
         </is>
       </c>
+      <c r="M81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5215,6 +5447,10 @@
 Étant donné l'export de vue simple, quand le fichier est ouvert, alors les métadonnées d'en-tête (nom de la vue, date d'export, source « HydroScope ») précisent le périmètre diffusé. --- EPIC 9 — Utilisateurs</t>
         </is>
       </c>
+      <c r="M82">
+        <f>SUMIF('Besoins testables'!$D:$D,$A82,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5272,6 +5508,7 @@
           <t>En tant qu'administrateur plateforme, je veux créer des comptes utilisateurs afin de permettre à chaque usager d'accéder à la plateforme.</t>
         </is>
       </c>
+      <c r="M83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5333,6 +5570,10 @@
 Étant donné la conformité RGPD (cookies / stockage local), quand une session est ouverte, alors aucun mot de passe ni donnée personnelle sensible n'est stocké côté navigateur.</t>
         </is>
       </c>
+      <c r="M84">
+        <f>SUMIF('Besoins testables'!$D:$D,$A84,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5398,6 +5639,10 @@
 Étant donné le changement de rôle d'un compte, quand il est enregistré, alors les nouveaux droits sont appliqués à la connexion suivante, sans privilège résiduel sur la session antérieure. --- EPIC 10 — Traçabilité</t>
         </is>
       </c>
+      <c r="M85">
+        <f>SUMIF('Besoins testables'!$D:$D,$A85,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5455,6 +5700,7 @@
           <t>En tant qu'administrateur plateforme, je veux restreindre finement l'accès aux données et aux fonctionnalités afin de limiter la consultation aux seuls droits autorisés.</t>
         </is>
       </c>
+      <c r="M86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5512,6 +5758,7 @@
           <t>En tant qu'administrateur plateforme, je veux adapter l'interface selon le profil de l'utilisateur afin d'afficher les fonctionnalités pertinentes pour chacun.</t>
         </is>
       </c>
+      <c r="M87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5569,6 +5816,7 @@
           <t>En tant qu'administrateur plateforme, je veux suivre les connexions des utilisateurs afin de surveiller l'utilisation de la plateforme.</t>
         </is>
       </c>
+      <c r="M88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5629,6 +5877,10 @@
 Étant donné un import suivi, quand il est enregistré, alors l'événement est visible dans le journal dans un délai conforme aux engagements contractuels, indépendamment du statut ultérieur des données.</t>
         </is>
       </c>
+      <c r="M89">
+        <f>SUMIF('Besoins testables'!$D:$D,$A89,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5694,6 +5946,10 @@
 Étant donné l'échec d'un calcul, quand il est journalisé, alors le motif est explicité, accessible à l'administrateur pour permettre la correction. --- *Périmètre MVP — Ce document référence le catalogue des indicateurs (38 indicateurs) et les référentiels (BVAEP, captages, PPE) fournis en données de référence pour la recette en Nouvelle-Calédonie. La liste des US couvertes correspond aux flags `MVP=TRUE` du fichier backlog.csv : 33 US au total pour les EPIC 6 à 10, dont 24 pour l'EPIC 6.* ---</t>
         </is>
       </c>
+      <c r="M90">
+        <f>SUMIF('Besoins testables'!$D:$D,$A90,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5746,6 +6002,7 @@
           <t>En tant qu'administrateur plateforme, je veux consulter le journal des actions afin de tracer les opérations effectuées sur la plateforme.</t>
         </is>
       </c>
+      <c r="M91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5803,6 +6060,7 @@
           <t>En tant qu'administrateur expert data, je veux consulter l'historique des modifications afin de suivre les changements.</t>
         </is>
       </c>
+      <c r="M92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5860,6 +6118,7 @@
           <t>En tant qu'administrateur expert data, je veux reconstituer un calcul afin de vérifier un résultat passé.</t>
         </is>
       </c>
+      <c r="M93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5912,6 +6171,7 @@
           <t>En tant qu'administrateur plateforme, je veux auditer les usages de la plateforme afin de contrôler les accès et de justifier les actions.</t>
         </is>
       </c>
+      <c r="M94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5964,6 +6224,7 @@
           <t>En tant qu'expert métier eau potable, je veux définir des seuils d'alerte afin de qualifier les valeurs des indicateurs et être averti des situations critiques.</t>
         </is>
       </c>
+      <c r="M95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6021,6 +6282,7 @@
           <t>En tant qu'expert métier eau potable, je veux détecter les dépassements de seuil afin d'anticiper les périodes de tension sur la ressource.</t>
         </is>
       </c>
+      <c r="M96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6081,6 +6343,10 @@
 Étant donné une série trop courte pour une tendance significative, quand elle est demandée, alors l'état « historique insuffisant » est affiché au lieu d'un résultat indicatif.</t>
         </is>
       </c>
+      <c r="M97">
+        <f>SUMIF('Besoins testables'!$D:$D,$A97,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6143,6 +6409,10 @@
           <t>Étant donné une règle de détection configurée (seuils US7.1, tendances US7.3), quand la valeur d'un indicateur sur un captage ou BVAEP franchit le critère de changement significatif, alors une alerte au changement est levée, datée et qualifiée. - Étant donné une alerte levée, quand je consulte son détail, alors la règle déclencheuse (indicateur, delta, période comparée, seuil) est exposée de façon explicite et reproductible. - Étant donné un captage/BVAEP avec une alerte active, quand je consulte sa fiche ou sa vue, alors les indicateurs ayant évolué sont mis en évidence (badge/teinte), sans aucune notification poussée (consultation seule). - Étant donné une vue présentant plusieurs signalements, quand ils coexistent, alors l'alerte au changement est distinguée du dépassement de seuil (US7.1) et de la tendance (US7.3). - Étant donné une alerte active, quand la valeur revient sous le critère ou la période de référence change, alors l'alerte est levée ou marquée « en résolution », sans message résiduel trompeur. - Étant donné le suivi d'un captage/BVAEP, quand je consulte l'historique, alors les alertes passées restent consultables (date, règle, état) sans être écrasées. - Étant donné une série trop courte ou non historisée, quand une alerte serait candidate, alors l'état « historique insuffisant » est affiché et aucune alerte due n'est levée. - Étant donné un profil habilité, quand une alerte est active ou configurée, alors la lecture respecte les droits (RBAC) et la configuration reste tracée (utilisateur, date).</t>
         </is>
       </c>
+      <c r="M98">
+        <f>SUMIF('Besoins testables'!$D:$D,$A98,'Besoins testables'!$O:$O)</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6200,6 +6470,7 @@
           <t>En tant qu'expert métier eau potable, je veux prioriser les territoires selon leur score de criticité afin de concentrer les actions sur les zones les plus sensibles.</t>
         </is>
       </c>
+      <c r="M99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6252,8 +6523,10 @@
           <t>En tant qu'expert métier eau potable, je veux utiliser l'aide à l'interprétation avancée.</t>
         </is>
       </c>
+      <c r="M100" s="2" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A1:L100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6265,7 +6538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N207"/>
+  <dimension ref="A1:O207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6355,6 +6628,11 @@
           <t>Scénario testable (complet)</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Point d'effort prestataire (1er niveau)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6397,7 +6675,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Acquisition</t>
@@ -6423,6 +6700,7 @@
           <t>Étant donné un administrateur expert data connecté, Quand il importe un fichier CSV conforme au modèle attendu (en-têtes, types, unités), Alors les données sont enregistrées dans la plateforme, Et un message de succès indique le nombre de lignes chargées, Et le jeu de données apparaît dans le catalogue comme donnée source.</t>
         </is>
       </c>
+      <c r="O2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6465,7 +6743,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Acquisition</t>
@@ -6491,6 +6768,7 @@
           <t>Étant donné un fichier au format SIG (Shapefile, GeoJSON), Quand il est importé, Alors les géométries sont validées et converties dans le système de coordonnées de référence de la plateforme, Et les enregistrements invalides sont rejetés avec leur motif.</t>
         </is>
       </c>
+      <c r="O3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6533,7 +6811,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Acquisition</t>
@@ -6559,6 +6836,7 @@
           <t>Étant donné un fichier contenant des doublons (même identifiant captage et même date), Quand l'import est lancé, Alors les doublons sont détectés et signalés, Et aucun doublon n'est enregistré sans validation explicite de l'administrateur.</t>
         </is>
       </c>
+      <c r="O4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6601,7 +6879,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Acquisition</t>
@@ -6627,6 +6904,7 @@
           <t>Étant donné un import volumineux ou long, Quand l'import est lancé, Alors il s'exécute de manière asynchrone avec un statut visible (en cours / terminé / échec), sans bloquer les autres actions de l'administrateur.</t>
         </is>
       </c>
+      <c r="O5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6669,7 +6947,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Acquisition</t>
@@ -6695,6 +6972,7 @@
           <t>Étant donné un fichier non conforme (extension non supportée, colonnes obligatoires manquantes), Quand l'administrateur tente l'import, Alors l'import est refusée et un message d'erreur explicite liste les anomalies détectées.</t>
         </is>
       </c>
+      <c r="O6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6767,6 +7045,7 @@
           <t>Étant donné une source de données fichier, Quand l'administrateur définit une planification (fréquence journalière, hebdomadaire, mensuelle, heure d'exécution), Alors l'import est exécuté automatiquement à l'échéance prévue, Et chaque exécution est tracée (date, heure, source, résultat, volumétrie). - Quand un import planifié échoue, Alors son statut passe à « échec », l'événement est journalisé avec le motif, Et les exécutions suivantes restent programmées. - Quand la planification est modifiée ou supprimée, Alors seules les nouvelles exécutions respectent la configuration courante, les exécutions déjà tracées restant inchangées. - Quand deux imports planifiés se chevauchent, Alors le système les sérialise ou refuse le chevauchement sans perte de données.</t>
         </is>
       </c>
+      <c r="O7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6839,6 +7118,7 @@
           <t>Étant donné un import planifié sans fichier source disponible à l'échéance, Alors l'exécution est signalée en échec avec un motif explicite, Et aucune donnée partielle ou vide n'est enregistrée.</t>
         </is>
       </c>
+      <c r="O8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6911,6 +7191,7 @@
           <t>Étant donné des données brutes hétérogènes (unités, formats de date, nomenclatures), Quand elles sont intégrées, Alors elles sont converties selon les règles de normalisation de la plateforme (unités de référence, dates ISO 8601, identifiants des référentiels), Et chaque transformation est documentée et tracée.</t>
         </is>
       </c>
+      <c r="O9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6983,6 +7264,7 @@
           <t>Étant donné une valeur référant à un captage ou un BVAEP, Quand la normalisation s'exécute, Alors la valeur est rattachée à l'objet correspondant du référentiel, Et toute valeur non rattachable est signalée en anomalie sans bloquer le reste du jeu.</t>
         </is>
       </c>
+      <c r="O10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7055,6 +7337,7 @@
           <t>Étant donné une valeur numérique hors plage ou un format inattendu, Quand la normalisation échoue pour cette ligne, Alors la ligne est marquée « non normalisée », Et le reste du jeu est traité sans blocage global. - Quand aucune règle de normalisation n'existe pour une colonne obligatoire, Alors l'import est refusée avec un message renvoyant vers la configuration de la source. - Quand un jeu de données normalisé est réimporté, Alors les mêmes règles produisent les mêmes valeurs (reproductibilité de la normalisation).</t>
         </is>
       </c>
+      <c r="O11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7127,6 +7410,7 @@
           <t>Étant donné un fichier CSV contenant 3 lignes invalides sur 100, Quand l'import est exécuté, Alors un rapport d'erreurs est généré listant les 3 lignes avec leur motif de rejet, Et les 97 lignes valides sont enregistrées. - Quand l'administrateur ouvre le rapport d'erreurs, Alors il voit pour chaque erreur le numéro de ligne, la valeur en cause et le motif (type, plage, rattachement référentiel, doublon).</t>
         </is>
       </c>
+      <c r="O12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7199,6 +7483,7 @@
           <t>Étant donné un fichier entièrement invalide, Quand aucun enregistrement ne passe les contrôles, Alors l'import est refusée dans sa globalité et aucun enregistrement n'est créé. - Quand un import se termine avec des rejets, Alors un message d'alerte informe l'administrateur du nombre d'enregistrements rejetés, avec un lien vers le rapport d'erreurs.</t>
         </is>
       </c>
+      <c r="O13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7271,6 +7556,7 @@
           <t>Étant donné un fichier corrigé après un rejet, Quand l'administrateur relance l'import, Alors seules les nouvelles anomalies sont signalées, les lignes précédemment corrigées n'apparaissant plus dans le rapport.</t>
         </is>
       </c>
+      <c r="O14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7343,6 +7629,7 @@
           <t>Étant donné un jeu de données déjà importé, Quand un nouvel import met à jour ce jeu, Alors une nouvelle version est créée, Et les versions antérieures sont intégralement conservées et consultables. - Quand une donnée est modifiée ou supprimée, Alors l'historisation conserve l'intégralité des versions antérieures : aucune valeur écrasée n'est perdue.</t>
         </is>
       </c>
+      <c r="O15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7415,6 +7702,7 @@
           <t>Étant donné une date de référence, Quand l'administrateur interroge l'historique, Alors il peut reconstituer l'état du jeu de données tel qu'il existait à cette date. - Quand une nouvelle version est enregistrée, Alors son horodatage, sa source et le traitement d'origine sont tracés. - Quand une opération de réécriture est demandée, Alors aucune donnée existante n'est écrasée sans création préalable d'une nouvelle version (aucune suppression destructive). ### EPIC 1bis — Catalogage des données</t>
         </is>
       </c>
+      <c r="O16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7487,6 +7775,7 @@
           <t>Étant donné un jeu de données intégré dans la plateforme, Quand l'administrateur l'enregistre dans le catalogue, Alors il reçoit un identifiant unique de catalogue, Et il devient visible et trouvable dans la liste du catalogue. - Quand un jeu de données est enregistré, Alors les champs obligatoires suivants sont renseignés et validés : nom, fournisseur, date de mise à jour, licence ; l'enregistrement est refusé tant qu'ils sont manquants.</t>
         </is>
       </c>
+      <c r="O17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7559,6 +7848,7 @@
           <t>Étant donné un identifiant de catalogue déjà utilisé, Quand l'administrateur tente d'enregistrer un autre jeu avec cet identifiant, Alors l'enregistrement est refusée et un message explicite s'affiche. - Quand un jeu de données enregistré est mis à jour (nouvel import), Alors la fiche du catalogue reste liée à la version courante du jeu.</t>
         </is>
       </c>
+      <c r="O18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7631,6 +7921,7 @@
           <t>Étant donné un jeu de données non encore intégré, Quand l'administrateur tente de l'enregistrer, Alors l'enregistrement est refusée : le catalogue ne référence que des données réellement disponibles dans la plateforme.</t>
         </is>
       </c>
+      <c r="O19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7703,6 +7994,7 @@
           <t>Étant donné un jeu de données du catalogue, Quand l'administrateur renseigne ses métadonnées, Alors les métadonnées obligatoires sont enregistrées : nom, fournisseur, date de mise à jour, licence ; Et le système refuse l'enregistrement tant qu'elles sont manquantes. - Quand des métadonnées descriptives sont saisies (origine, couverture spatiale et temporelle, unités, fréquence de mise à jour, contact), Alors elles sont structurées selon un schéma commun et affichées sur la fiche du jeu de données.</t>
         </is>
       </c>
+      <c r="O20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7775,6 +8067,7 @@
           <t>Étant donné un jeu de données géographique, Quand ses métadonnées sont saisies, Alors le système de coordonnées et la couverture spatiale (communes, BVAEP concernés) sont documentés. - Quand des métadonnées sont enregistrées, Alors la date et l'auteur de la saisie sont tracés.</t>
         </is>
       </c>
+      <c r="O21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7847,6 +8140,7 @@
           <t>Étant donné une licence non autorisée ou une date de mise à jour future, Quand l'enregistrement est tenté, Alors il est refusé avec un message d'erreur explicite.</t>
         </is>
       </c>
+      <c r="O22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7889,7 +8183,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -7915,6 +8208,7 @@
           <t>Étant donné un jeu de données du catalogue, Quand l'utilisateur ouvre sa fiche, Alors il voit son nom, son fournisseur, sa date de mise à jour, sa licence, sa couverture spatiale et temporelle, et son type (donnée source ou donnée dérivée). - Quand l'utilisateur consulte la fiche, Alors il voit la structure du jeu (champs, types, unités) et, si disponible, un aperçu du contenu.</t>
         </is>
       </c>
+      <c r="O23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7957,7 +8251,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -7983,6 +8276,7 @@
           <t>Étant donné un jeu de données dérivé, Quand sa fiche est consultée, Alors elle affiche les données sources et les traitements dont il provient.</t>
         </is>
       </c>
+      <c r="O24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8025,7 +8319,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -8051,6 +8344,7 @@
           <t>Étant donné un jeu de données sans licence renseignée, Quand sa fiche est consultée, Alors la mention « licence non renseignée » est affichée (aucune valeur par défaut trompeuse). - Quand la fiche est consultée depuis le catalogue, Alors l'utilisateur voit les métadonnées de qualité associées (EPIC 2) si elles existent.</t>
         </is>
       </c>
+      <c r="O25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8093,7 +8387,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -8119,6 +8412,7 @@
           <t>Étant donné un indicateur dérivé, Quand l'utilisateur ouvre sa page de relations, Alors il voit un graphe reliant l'indicateur à ses données sources et aux traitements intermédiaires. - Quand l'utilisateur clique sur un nœud du graphe (jeu de données source, traitement), Alors les métadonnées correspondantes sont affichées.</t>
         </is>
       </c>
+      <c r="O26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8161,7 +8455,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -8187,6 +8480,7 @@
           <t>Étant donné un indicateur calculé sur des données historisées, Quand le graphe est affiché, Alors la version ou la période des données utilisées pour le calcul courant est précisée.</t>
         </is>
       </c>
+      <c r="O27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8229,7 +8523,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -8255,6 +8548,7 @@
           <t>Étant donné un indicateur sans dépendance déclarée, Quand la page est ouverte, Alors un message indique l'absence de relations tracées plutôt qu'un graphe vide. - Quand l'indicateur est recalculé sur de nouvelles données, Alors le graphe reflète les relations de la version de calcul la plus récente.</t>
         </is>
       </c>
+      <c r="O28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8327,6 +8621,7 @@
           <t>Étant donné un import de fichier réussi, Quand le traitement se termine, Alors une entrée de catalogue est créée ou mise à jour automatiquement, sans saisie manuelle.</t>
         </is>
       </c>
+      <c r="O29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8399,6 +8694,7 @@
           <t>Étant donné un jeu de données déjà catalogué, Quand un import le met à jour, Alors sa fiche de catalogue est actualisée (date de mise à jour, version courante) sans création de doublon.</t>
         </is>
       </c>
+      <c r="O30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8471,6 +8767,7 @@
           <t>Étant donné un import en échec, Quand le traitement se termine, Alors aucune entrée de catalogue n'est créée, Et l'événement est tracé. - Quand une entrée est créée automatiquement, Alors les métadonnées minimales (nom, fournisseur, date de mise à jour) sont déduites de l'import et marquées « générées automatiquement ».</t>
         </is>
       </c>
+      <c r="O31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8543,6 +8840,7 @@
           <t>Étant donné un import sans identifiant de jeu identifiable, Quand l'alimentation du catalogue est tentée, Alors l'import est signalé en échec partiel avec le motif.</t>
         </is>
       </c>
+      <c r="O32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8615,6 +8913,7 @@
           <t>Étant donné un indicateur défini dans le référentiel (US3.5), Quand il est enregistré dans le catalogue, Alors il apparaît avec le type « donnée dérivée », distinct des données sources. - Quand la fiche de l'indicateur est consultée, Alors elle indique qu'il s'agit d'une donnée dérivée et renvoie vers sa définition et sa méthode de calcul.</t>
         </is>
       </c>
+      <c r="O33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8687,6 +8986,7 @@
           <t>Étant donné un enregistrement sans lien vers une donnée source ou un traitement, Quand il est tenté, Alors il est refusé : tout indicateur dérivé référence au moins une donnée source ou un traitement.</t>
         </is>
       </c>
+      <c r="O34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8759,6 +9059,7 @@
           <t>Étant donné un indicateur non défini dans le référentiel, Quand l'administrateur tente de l'enregistrer, Alors l'enregistrement est refusé avec un message renvoyant vers la définition de l'indicateur (US3.5). - Quand un indicateur dérivé est recalculé, Alors la version cataloguée est mise à jour, Et la traçabilité du calcul (date, version de la méthode, données utilisées) est conservée. ### EPIC 2 — Qualité des données</t>
         </is>
       </c>
+      <c r="O35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8801,7 +9102,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -8827,6 +9127,7 @@
           <t>Étant donné un jeu de données avec des règles de contrôle définies (bornes min/max, plages attendues), Quand une valeur sort de la plage attendue, Alors l'anomalie est détectée et enregistrée avec le jeu de données, la ligne, la valeur et la règle violée. - Quand la détection est exécutée, Alors un rapport liste les valeurs aberrantes avec leur motif, sans modifier les données d'origine.</t>
         </is>
       </c>
+      <c r="O36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8869,7 +9170,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -8895,6 +9195,7 @@
           <t>Étant donné une valeur aberrante détectée et validée comme erronée par l'administrateur, Alors elle est exclue des traitements ou marquée non fiable, tout en restant disponible dans l'historique.</t>
         </is>
       </c>
+      <c r="O37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8937,7 +9238,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -8963,6 +9263,7 @@
           <t>Étant donné une valeur signalée à tort (faux positif), Quand l'administrateur la blanchit, Alors le motif du blanchiment est documenté et tracé.</t>
         </is>
       </c>
+      <c r="O38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9005,7 +9306,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9031,6 +9331,7 @@
           <t>Étant donné un jeu sans règles de détection configurées, Quand le contrôle est exécuté, Alors aucune valeur aberrante n'est signalée et le jeu est qualifié « non contrôlé ».</t>
         </is>
       </c>
+      <c r="O39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9073,7 +9374,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9099,6 +9399,7 @@
           <t>Étant donné un jeu de données avec des champs obligatoires définis, Quand le taux de complétude est calculé, Alors il correspond au pourcentage de valeurs renseignées sur les valeurs attendues, par champ et par jeu, Et le résultat est stocké comme métadonnée de qualité. - Quand un taux est calculé, Alors la période et la version du jeu de données utilisées pour le calcul sont précisées.</t>
         </is>
       </c>
+      <c r="O40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9141,7 +9442,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9167,6 +9467,7 @@
           <t>Étant donné un seuil de complétude configuré (par défaut 95 %), Quand le taux calculé est inférieur au seuil, Alors le jeu est marqué comme sous le seuil, Et l'information est reportée sur sa fiche qualité. - Quand un jeu est mis à jour (nouvel import, corrections), Alors le taux est recalculé sur la dernière version, sans perte des taux historiques. - Quand le taux de complétude d'un jeu sert au calcul d'un indicateur (EPIC 4), Alors il est exploitable de façon automatisée (filtrage ou marquage du résultat).</t>
         </is>
       </c>
+      <c r="O41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9209,7 +9510,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9235,6 +9535,7 @@
           <t>Étant donné les critères de fiabilité définis (source, méthode de production, complétude, fréquence de mise à jour), Quand la fiabilité d'un jeu de données est évaluée, Alors une classe de fiabilité (élevée, moyenne, faible) lui est attribuée selon des règles documentées. - Quand une classe de fiabilité est attribuée, Alors la règle et les critères utilisés sont tracés.</t>
         </is>
       </c>
+      <c r="O42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9277,7 +9578,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9303,6 +9603,7 @@
           <t>Étant donné un jeu dont la qualité évolue (nouvel import, corrections), Quand la fiabilité est réévaluée, Alors la classe est recalculée, Et l'évolution est conservée dans l'historique des indicateurs de qualité.</t>
         </is>
       </c>
+      <c r="O43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9345,7 +9646,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9371,6 +9671,7 @@
           <t>Étant donné un jeu sans métadonnées de qualité renseignées, Quand l'évaluation est demandée, Alors aucune classe n'est attribuée : le jeu est qualifié « fiabilité non évaluée » (pas de note par défaut trompeuse). - Quand une classe de fiabilité est disponible, Alors elle est exploitable par les traitements ultérieurs (filtrage, affichage différencié).</t>
         </is>
       </c>
+      <c r="O44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9413,7 +9714,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9439,6 +9739,7 @@
           <t>Étant donné un jeu de données contrôlé, Quand l'administrateur associe des métadonnées de qualité, Alors il renseigne : date du dernier contrôle, règles appliquées, résultats (anomalies, taux de complétude, fiabilité) et statut de validation. - Quand des métadonnées de qualité sont enregistrées, Alors elles sont visibles sur la fiche qualité du jeu de données.</t>
         </is>
       </c>
+      <c r="O45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9481,7 +9782,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9507,6 +9807,7 @@
           <t>Étant donné un contrôle automatique, Quand il s'exécute, Alors ses résultats alimentent les métadonnées de qualité sans saisie manuelle, Et l'horodatage du contrôle est tracé.</t>
         </is>
       </c>
+      <c r="O46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9549,7 +9850,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>Qualification</t>
@@ -9575,6 +9875,7 @@
           <t>Étant donné un jeu de données non intégré dans la plateforme, Quand l'administrateur tente d'ajouter des métadonnées de qualité, Alors l'opération est refusée avec un message explicite. - Quand l'administrateur consulte la fiche qualité, Alors il voit un résumé : date du dernier contrôle, classe de fiabilité, taux de complétude, nombre d'anomalies ouvertes. ### EPIC 3 — Référentiels</t>
         </is>
       </c>
+      <c r="O47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9617,7 +9918,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9643,6 +9943,7 @@
           <t>Étant donné le référentiel des BVAEP, Quand l'administrateur crée un bassin versant d'alimentation en eau potable, Alors il renseigne au minimum : identifiant, nom, géométrie, communes et captages rattachés, Et le BVAEP devient utilisable dans les agrégations et sur la carte. - Quand l'administrateur modifie la géométrie ou le périmètre d'un BVAEP, Alors la modification est enregistrée avec sa date, Et les données historiques restent rattachées à l'ancien périmètre (cohérence temporelle).</t>
         </is>
       </c>
+      <c r="O48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -9685,7 +9986,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9711,6 +10011,7 @@
           <t>Étant donné un identifiant de BVAEP déjà utilisé ou une géométrie invalide, Quand la création ou la modification est tentée, Alors elle est refusée avec un message explicite. - Quand l'administrateur consulte la liste des BVAEP, Alors il voit l'identifiant, le nom, les communes et le nombre de captages rattachés.</t>
         </is>
       </c>
+      <c r="O49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9753,7 +10054,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9779,6 +10079,7 @@
           <t>Étant donné un BVAEP auquel des données ou des captages sont rattachés, Quand l'administrateur tente de le supprimer, Alors la suppression est refusée tant qu'aucun réaffectement explicite n'a été effectué.</t>
         </is>
       </c>
+      <c r="O50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -9821,7 +10122,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9847,6 +10147,7 @@
           <t>Étant donné le référentiel des captages, Quand l'administrateur crée un captage, Alors il renseigne au minimum : identifiant, nom, commune, coordonnées et BVAEP de rattachement, Et le captage apparaît dans le référentiel et sur la carte. - Quand un captage est rattaché à un BVAEP, Alors la cohérence du rattachement est vérifiée (position dans le bassin ou rattachement explicite justifié), Et toute incohérence est signalée. - Quand l'administrateur modifie un captage (localisation, rattachement, statut), Alors la version précédente est conservée pour la reconstitution historique. - Quand la fiche du captage est consultée, Alors elle affiche ses données de qualité (EPIC 2) et les périmètres de protection (PPE) associés s'ils sont renseignés.</t>
         </is>
       </c>
+      <c r="O51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9889,7 +10190,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9915,6 +10215,7 @@
           <t>Étant donné un identifiant de captage déjà utilisé, Quand la création est tentée, Alors elle est refusée avec un message explicite.</t>
         </is>
       </c>
+      <c r="O52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9957,7 +10258,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -9983,6 +10283,7 @@
           <t>Étant donné le référentiel de la maille H3, Quand l'administrateur définit les résolutions utilisées par la plateforme, Alors la configuration est enregistrée et documentée, Et elle sert de référence aux agrégations. - Quand l'administrateur consulte la maille, Alors il voit la grille H3 superposée à la carte avec ses cellules identifiées.</t>
         </is>
       </c>
+      <c r="O53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -10025,7 +10326,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10051,6 +10351,7 @@
           <t>Étant donné des objets du référentiel (captages, BVAEP, communes), Quand leur rattachement à la maille H3 est calculé, Alors chaque objet est associé aux cellules qu'il intersecte, Et le résultat est tracé pour garantir la cohérence des agrégations.</t>
         </is>
       </c>
+      <c r="O54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10093,7 +10394,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10119,6 +10419,7 @@
           <t>Étant donné une modification de la résolution configurée, Quand elle est enregistrée, Alors les agrégations existantes restent reproductibles et les données historiques ne sont pas altérées.</t>
         </is>
       </c>
+      <c r="O55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -10161,7 +10462,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10187,6 +10487,7 @@
           <t>Étant donné une résolution non supportée, Quand l'administrateur tente de la configurer, Alors l'opération est refusée avec la liste des résolutions disponibles.</t>
         </is>
       </c>
+      <c r="O56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -10229,7 +10530,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10255,6 +10555,7 @@
           <t>Étant donné le référentiel des indicateurs, Quand l'administrateur définit un indicateur, Alors il renseigne au minimum : nom, description, finalité, unité, échelle spatiale (captage, BVAEP, maille H3) et temporelle, méthode de calcul et liens vers les données sources ; l'enregistrement est refusé tant que ces éléments sont manquants. - Quand l'indicateur est enregistré, Alors il devient calculable par le moteur (EPIC 4), affichable dans le catalogue et exploitable par la carte. - Quand l'administrateur modifie la méthode de calcul d'un indicateur, Alors une nouvelle version de la définition est créée, Et les versions antérieures restent consultables.</t>
         </is>
       </c>
+      <c r="O57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10297,7 +10598,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10323,6 +10623,7 @@
           <t>Étant donné un indicateur avec des seuils, Quand ils sont définis, Alors ils sont enregistrés avec l'indicateur et disponibles pour la qualification des valeurs.</t>
         </is>
       </c>
+      <c r="O58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10365,7 +10666,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>Structuration</t>
@@ -10391,6 +10691,7 @@
           <t>Étant donné un indicateur déjà défini sous le même nom ou le même identifiant, Quand la définition est tentée, Alors elle est refusée avec un message explicite. ### EPIC 4 — Calcul d'indicateurs</t>
         </is>
       </c>
+      <c r="O59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10463,6 +10764,7 @@
           <t>Étant donné un indicateur défini (US3.5) et ses données sources cataloguées et qualifiées, Quand le calcul est exécuté, Alors les valeurs produites respectent la méthode définie (moyenne, médiane, somme, fréquence, occurrence), Et le résultat est stocké avec la date de calcul, la version de la définition et les versions des données utilisées.</t>
         </is>
       </c>
+      <c r="O60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -10535,6 +10837,7 @@
           <t>Étant donné un calcul reposant sur des données manquantes ou sous le seuil de complétude, Quand le résultat est produit, Alors il est marqué « non fiable » ou non calculé selon les règles de l'indicateur.</t>
         </is>
       </c>
+      <c r="O61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10607,6 +10910,7 @@
           <t>Étant donné un calcul en échec, Quand il se termine, Alors aucune valeur n'est publiée, Et l'échec est tracé avec son motif. - Quand le calcul est relancé après correction des données, Alors le résultat est recalculé et la nouvelle exécution est tracée (reproductibilité).</t>
         </is>
       </c>
+      <c r="O62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10679,6 +10983,7 @@
           <t>Étant donné un indicateur sans méthode complète ou sans données sources, Quand le calcul est demandé, Alors il est refusé avec un message explicite.</t>
         </is>
       </c>
+      <c r="O63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10751,6 +11056,7 @@
           <t>Étant donné des valeurs à l'échelle captage ou maille H3, Quand l'agrégation à l'échelle du BVAEP est exécutée, Alors une valeur synthétique est produite pour chaque bassin versant selon la règle d'agrégation définie (somme, moyenne, moyenne pondérée), Et la règle utilisée est tracée. - Quand le résultat d'agrégation est produit, Alors il est accompagné de la liste des captages pris en compte et du taux de complétude associé.</t>
         </is>
       </c>
+      <c r="O64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10823,6 +11129,7 @@
           <t>Étant donné un captage non rattaché à un BVAEP, Quand l'agrégation est exécutée, Alors il est exclu du calcul et signalé dans les anomalies.</t>
         </is>
       </c>
+      <c r="O65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10895,6 +11202,7 @@
           <t>Étant donné une évolution du périmètre d'un BVAEP, Quand l'agrégation est exécutée sur une période passée, Alors elle utilise la version du périmètre applicable à cette période (cohérence historique).</t>
         </is>
       </c>
+      <c r="O66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -10967,6 +11275,7 @@
           <t>Étant donné un indicateur sans règle d'agrégation spatiale définie, Quand l'agrégation à l'échelle BV est demandée, Alors elle est refusée avec un message explicite.</t>
         </is>
       </c>
+      <c r="O67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -11039,6 +11348,7 @@
           <t>Étant donné des données historisées (US1.6), Quand l'agrégation temporelle (mensuelle, annuelle, pluriannuelle) est exécutée, Alors les séries consolidées sont produites sur les périodes demandées, Et les données sous-jacentes restent disponibles.</t>
         </is>
       </c>
+      <c r="O68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -11111,6 +11421,7 @@
           <t>Étant donné une période contenant des données manquantes, Quand le résultat est produit, Alors le taux de couverture de la période est indiqué, Et le résultat est marqué si le seuil de complétude n'est pas atteint. - Quand la même agrégation est relancée sur la même période et les mêmes données, Alors le résultat est identique (reproductibilité des calculs).</t>
         </is>
       </c>
+      <c r="O69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -11183,6 +11494,7 @@
           <t>Étant donné une période demandée dépassant l'historique disponible, Quand l'agrégation est exécutée, Alors elle est limitée à l'historique existant et l'écart est signalé, ou refusée si aucune donnée ne couvre la période. - Quand un indicateur est produit à plusieurs granularités temporelles, Alors le périmètre de calcul (données incluses, période couverte) est documenté pour garantir la comparabilité des séries.</t>
         </is>
       </c>
+      <c r="O70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -11225,7 +11537,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -11251,6 +11562,7 @@
           <t>Étant donné l'interface de calcul d'un indicateur, Quand l'administrateur applique des filtres (période, source, qualité, territoire : captage, BVAEP, commune), Alors seules les valeurs répondant aux filtres sont utilisées dans le calcul, Et les filtres appliqués sont affichés à l'écran. - Quand l'administrateur exclut les données de qualité insuffisante (fiabilité faible, anomalies, sous le seuil de complétude), Alors elles sont exclues du calcul, Et l'option d'exclusion est visible dans l'interface. - Quand les filtres sont modifiés, Alors le calcul est relancé sur le nouveau périmètre, Et aucun résultat obsolète n'est affiché sans mention.</t>
         </is>
       </c>
+      <c r="O71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -11293,7 +11605,6 @@
           <t>Gestion des données &amp; catalogue</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -11319,6 +11630,7 @@
           <t>Étant donné une combinaison de filtres ne sélectionnant aucune donnée, Quand le calcul est demandé, Alors il est refusé avec le message « aucun jeu de données ne correspond aux filtres appliqués ». - Quand l'administrateur consulte la configuration du calcul, Alors il voit un résumé des critères retenus (période, sources, territoires, seuil de qualité) avant exécution.</t>
         </is>
       </c>
+      <c r="O72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -11361,7 +11673,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -11387,6 +11698,7 @@
           <t>Étant donné la plateforme opérationnelle avec des données BVAEP et captages chargées, quand je consulte la vue « Carte », alors une carte interactive s'affiche (fond Cartographique par défaut) avec les objets du périmètre positionnés.</t>
         </is>
       </c>
+      <c r="O73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -11429,7 +11741,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -11455,6 +11766,7 @@
           <t>Étant donné une carte affichée, quand je me déplace (pan) ou je zoome, alors l'emprise se met à jour et les objets pertinents apparaissent, sans rechargement de la page.</t>
         </is>
       </c>
+      <c r="O74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -11497,7 +11809,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -11523,6 +11834,7 @@
           <t>Étant donné un objet visible (BVAEP, captage, PPE), quand je le survole, alors une infobulle présente son nom et son identifiant.</t>
         </is>
       </c>
+      <c r="O75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -11565,7 +11877,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -11591,6 +11902,7 @@
           <t>Étant donné une zone sans donnée dans l'emprise, quand la carte est rendue, alors le périmètre reste lisible avec un libellé explicite (pas de fond vide ambigu).</t>
         </is>
       </c>
+      <c r="O76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -11663,6 +11975,7 @@
           <t>Étant donné un indicateur sélectionné dans le volet indicateurs, quand je l'applique à la carte, alors les unités sont colorées selon les classes de valeurs de l'indicateur, avec une légende affichant la plage et les couleurs.</t>
         </is>
       </c>
+      <c r="O77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -11735,6 +12048,7 @@
           <t>Étant donné une unité sans valeur pour l'indicateur, quand la carte est rendue, alors cette unité est affectée à une classe « sans donnée » distincte, hors plage de valeurs.</t>
         </is>
       </c>
+      <c r="O78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -11807,6 +12121,7 @@
           <t>Étant donné un indicateur calculé ou recalculé, quand je rafraîchis le rendu cartographique, alors les couleurs correspondent aux nouvelles valeurs sans référence obsolète.</t>
         </is>
       </c>
+      <c r="O79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -11879,6 +12194,7 @@
           <t>Étant donné un changement d'indicateur (via Famille → Thème → Groupe), quand je bascule, alors la légende et les couleurs correspondent immédiatement au nouvel indicateur en conservant la sélection courante.</t>
         </is>
       </c>
+      <c r="O80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -11921,7 +12237,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -11947,6 +12262,7 @@
           <t>Étant donné la carte, quand j'utilise les contrôles de zoom et le pan, alors l'emprise évolue et les unités affichées sont recalculées de façon synchrone.</t>
         </is>
       </c>
+      <c r="O81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -11989,7 +12305,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12015,6 +12330,7 @@
           <t>Étant donné une sélection ou des filtres actifs, quand je navigue sur la carte, alors la sélection et les filtres ne sont ni réinitialisés ni altérés.</t>
         </is>
       </c>
+      <c r="O82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -12057,7 +12373,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12083,6 +12398,7 @@
           <t>Étant donné une navigation avancée, quand j'actionne la réinitialisation de la vue, alors l'emprise revient au périmètre par défaut en conservant les filtres utilisateur.</t>
         </is>
       </c>
+      <c r="O83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -12125,7 +12441,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12151,6 +12466,7 @@
           <t>Étant donné un changement d'échelle, quand les unités deviennent trop nombreuses à l'écran, alors la carte propose un regroupement lisible (agrégation visuelle) sans perte de données.</t>
         </is>
       </c>
+      <c r="O84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -12223,6 +12539,7 @@
           <t>Étant donné un indicateur à données historisées, quand je consulte son graphique temporel, alors une série chronologique est tracée avec unité, dates et période affichées.</t>
         </is>
       </c>
+      <c r="O85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -12295,6 +12612,7 @@
           <t>Étant donné plusieurs unités sélectionnées (captages et/ou BVAEP), quand le graphique temporel est affiché, alors chaque série est identifiée et distinguée par une palette de couleurs cohérente avec la carte.</t>
         </is>
       </c>
+      <c r="O86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -12367,6 +12685,7 @@
           <t>Étant donné une période sans mesure, quand elle appartient à la série, alors elle apparaît comme une lacune explicite (valeur indisponible), jamais remplacée par un zéro.</t>
         </is>
       </c>
+      <c r="O87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -12439,6 +12758,7 @@
           <t>Étant donné un point de la série, quand je le survole, alors une infobulle affiche la date et la valeur de l'indicateur.</t>
         </is>
       </c>
+      <c r="O88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -12481,7 +12801,6 @@
           <t>Cartographie &amp; exploration &gt; Fiches &amp; synthèse territoriale</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12507,6 +12826,7 @@
           <t>Étant donné une fiche territoire (commune, BVAEP ou bassin versant), quand je la consulte, alors elle présente le périmètre décrit, les unités de gestion associées et les indicateurs disponibles.</t>
         </is>
       </c>
+      <c r="O89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -12549,7 +12869,6 @@
           <t>Cartographie &amp; exploration &gt; Fiches &amp; synthèse territoriale</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12575,6 +12894,7 @@
           <t>Étant donné une fiche territoire générée, quand elle est affichée, alors son contenu est strictement issu des données et indicateurs produits, sans ajout interprétatif ni classement/priorisation.</t>
         </is>
       </c>
+      <c r="O90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -12617,7 +12937,6 @@
           <t>Cartographie &amp; exploration &gt; Fiches &amp; synthèse territoriale</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12643,6 +12962,7 @@
           <t>Étant donné une unité cartographique, quand je l'active (clic ou sélection), alors je peux ouvrir sa fiche territoire depuis la carte.</t>
         </is>
       </c>
+      <c r="O91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -12685,7 +13005,6 @@
           <t>Cartographie &amp; exploration &gt; Fiches &amp; synthèse territoriale</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -12711,6 +13030,7 @@
           <t>Étant donné une donnée source mise à jour, quand la fiche est consultée, alors elle reflète la dernière version sans action manuelle.</t>
         </is>
       </c>
+      <c r="O92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -12783,6 +13103,7 @@
           <t>Étant donné une échelle active (captages ou BVAEP), quand je bascule l'échelle, alors la carte affiche immédiatement les unités de la nouvelle échelle sur la même emprise.</t>
         </is>
       </c>
+      <c r="O93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -12855,6 +13176,7 @@
           <t>Étant donné des sélections distinctes Captages et Bassins versants, quand j'alterne les échelles, alors chaque sélection est rappelée indépendamment (les types d'unités ne sont pas mélangés).</t>
         </is>
       </c>
+      <c r="O94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -12927,6 +13249,7 @@
           <t>Étant donné un indicateur applicable aux deux échelles, quand je bascule, alors la valeur affichée correspond à l'agrégation de l'échelle active (globale pour un BVAEP, ponctuelle pour un captage).</t>
         </is>
       </c>
+      <c r="O95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -12999,6 +13322,7 @@
           <t>Étant donné le compteur d'unités, quand je bascule d'échelle, alors il reflète immédiatement le nombre d'unités sélectionnées à la nouvelle échelle.</t>
         </is>
       </c>
+      <c r="O96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -13041,7 +13365,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13067,6 +13390,7 @@
           <t>Étant donné une sélection en cours, quand la vue est chargée, alors un compteur affiche le nombre d'unités sélectionnées, au format « X captages · Y bassins versants ».</t>
         </is>
       </c>
+      <c r="O97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -13109,7 +13433,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13135,6 +13458,7 @@
           <t>Étant donné une action d'ajout ou de retrait de sélection, quand elle est validée, alors le compteur se met à jour en temps réel.</t>
         </is>
       </c>
+      <c r="O98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -13177,7 +13501,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13203,6 +13526,7 @@
           <t>Étant donné une sélection vide, quand la vue est affichée, alors le compteur est à 0 avec un message invitant à sélectionner (aucune ambiguïté entre « rien » et « tout »).</t>
         </is>
       </c>
+      <c r="O99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -13245,7 +13569,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13271,6 +13594,7 @@
           <t>Étant donné la carte, les listes et le compteur, quand une sélection est modifiée, alors ils restent cohérents entre eux.</t>
         </is>
       </c>
+      <c r="O100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -13313,7 +13637,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13339,6 +13662,7 @@
           <t>Étant donné la zone de recherche, quand je saisis au moins deux caractères, alors des suggestions s'affichent pour : communes, provinces, captages, BVAEP et presets « Top 10 ».</t>
         </is>
       </c>
+      <c r="O101" s="2" t="n"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -13381,7 +13705,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13407,6 +13730,7 @@
           <t>Étant donné un nom saisi, quand la recherche ignore la casse et les accents, alors les résultats attendus sont retrouvés.</t>
         </is>
       </c>
+      <c r="O102" s="2" t="n"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -13449,7 +13773,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13475,6 +13798,7 @@
           <t>Étant donné le choix d'une suggestion commune ou province, quand je valide, alors la carte se centre sur l'entité et la sélection est restreinte à son périmètre (filtre géographique).</t>
         </is>
       </c>
+      <c r="O103" s="2" t="n"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -13517,7 +13841,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13543,6 +13866,7 @@
           <t>Étant donné une recherche sans résultat, quand elle est exécutée, alors un message « Aucun résultat » est affiché, sans rechargement ni erreur.</t>
         </is>
       </c>
+      <c r="O104" s="2" t="n"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -13585,7 +13909,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13611,6 +13934,7 @@
           <t>Étant donné plusieurs facettes (commune, province, type d'unité, indicateur), quand je les cumule, alors la sélection résultante est la combinaison des critères définie (intersection des filtres).</t>
         </is>
       </c>
+      <c r="O105" s="2" t="n"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -13653,7 +13977,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13679,6 +14002,7 @@
           <t>Étant donné un filtre et une sélection manuelle combinés, quand la vue est rendue, alors la carte, les listes et le compteur reflètent exactement la même combinaison.</t>
         </is>
       </c>
+      <c r="O106" s="2" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -13721,7 +14045,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13747,6 +14070,7 @@
           <t>Étant donné des facettes cumulées méthodologiquement incompatibles, quand je tente de les cumuler, alors le système présente un état « filtre incompatible » explicite, sans ambiguïté.</t>
         </is>
       </c>
+      <c r="O107" s="2" t="n"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -13789,7 +14113,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13815,6 +14138,7 @@
           <t>Étant donné l'état courant des facettes, quand je quitte puis reviens sur la vue, alors l'état est restauré ou clairement signalé comme non conservé.</t>
         </is>
       </c>
+      <c r="O108" s="2" t="n"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -13857,7 +14181,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13883,6 +14206,7 @@
           <t>Étant donné au moins un filtre actif, quand la vue s'affiche, alors une puce (chip) portant le libellé du filtre est visible.</t>
         </is>
       </c>
+      <c r="O109" s="2" t="n"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -13925,7 +14249,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -13951,6 +14274,7 @@
           <t>Étant donné plusieurs filtres cumulés, quand ils sont tous appliqués, alors une puce par filtre est affichée, sans doublon ni filtre invisible.</t>
         </is>
       </c>
+      <c r="O110" s="2" t="n"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -13993,7 +14317,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14019,6 +14342,7 @@
           <t>Étant donné une puce active, quand je clique sur sa croix de désélection, alors le filtre est retiré et toutes les vues (carte, liste, graphiques) se mettent à jour.</t>
         </is>
       </c>
+      <c r="O111" s="2" t="n"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -14061,7 +14385,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14087,6 +14410,7 @@
           <t>Étant donné l'ensemble des puces, quand je les retire une à une, alors la sélection initiale est progressivement restituée jusqu'au retour à l'état de départ.</t>
         </is>
       </c>
+      <c r="O112" s="2" t="n"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -14129,7 +14453,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14155,6 +14478,7 @@
           <t>Étant donné la zone des presets, quand je choisis « Top 10 les plus exposés » (et les variantes : moins exposés), alors la sélection et la liste affichent les dix unités calculées selon la règle du preset.</t>
         </is>
       </c>
+      <c r="O113" s="2" t="n"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -14197,7 +14521,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14223,6 +14546,7 @@
           <t>Étant donné un preset appliqué, quand la carte et les listes sont rendues, alors les dix unités sont identifiées dans les vues et cohérentes entre elles.</t>
         </is>
       </c>
+      <c r="O114" s="2" t="n"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -14265,7 +14589,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14291,6 +14614,7 @@
           <t>Étant donné une sélection utilisateur préalable, quand j'applique un preset, alors l'application du preset est explicite (remplacement ou superposition selon la règle définie), jamais silencieuse.</t>
         </is>
       </c>
+      <c r="O115" s="2" t="n"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -14333,7 +14657,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14359,6 +14682,7 @@
           <t>Étant donné un preset actif, quand je le retire, alors la sélection antérieure est restituée telle qu'elle était avant l'application.</t>
         </is>
       </c>
+      <c r="O116" s="2" t="n"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -14401,7 +14725,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14427,6 +14750,7 @@
           <t>Étant donné une unité non classable par la règle du preset, quand elle n'est pas retenue, alors elle n'est pas exclue silencieusement et reste consultable.</t>
         </is>
       </c>
+      <c r="O117" s="2" t="n"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -14469,7 +14793,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14495,6 +14818,7 @@
           <t>Étant donné une facette cochée dans le sélecteur, quand je la décoche, alors le filtre ou la sélection correspondant(e) est retiré(e) et toutes les vues se mettent à jour.</t>
         </is>
       </c>
+      <c r="O118" s="2" t="n"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -14537,7 +14861,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14563,6 +14886,7 @@
           <t>Étant donné une facette décochée, quand je la décoche à nouveau, alors rien ne change (comportement idempotent, sans erreur).</t>
         </is>
       </c>
+      <c r="O119" s="2" t="n"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -14605,7 +14929,6 @@
           <t>Cartographie &amp; exploration &gt; Outils d'exploration</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14631,6 +14954,7 @@
           <t>Étant donné un filtre retiré par décochage, quand je le ré-applique, alors le résultat correspond au résultat initial (pas de dérive de l'état).</t>
         </is>
       </c>
+      <c r="O120" s="2" t="n"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -14673,7 +14997,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14699,6 +15022,7 @@
           <t>Étant donné une liste de captages ou de BVAEP, quand je clique une unité, alors elle est sélectionnée ; au second clic, elle est désélectionnée.</t>
         </is>
       </c>
+      <c r="O121" s="2" t="n"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -14741,7 +15065,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14767,6 +15090,7 @@
           <t>Étant donné une unité sélectionnée, quand je la retire via sa puce ou son bouton dédié, alors elle est retirée de la sélection et les autres unités restent intactes.</t>
         </is>
       </c>
+      <c r="O122" s="2" t="n"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -14809,7 +15133,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14835,6 +15158,7 @@
           <t>Étant donné une sélection en cours, quand j'ajoute une unité individuelle, alors le compteur et la carte intègrent l'unité sans réinitialiser le reste.</t>
         </is>
       </c>
+      <c r="O123" s="2" t="n"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -14877,7 +15201,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14903,6 +15226,7 @@
           <t>Étant donné une unité retirée, quand un graphique est affiché, alors l'unité n'apparaît plus dans les séries renvoyées.</t>
         </is>
       </c>
+      <c r="O124" s="2" t="n"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -14945,7 +15269,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -14971,6 +15294,7 @@
           <t>Étant donné des sélections distinctes de captages et de BVAEP, quand je passe d'une échelle à l'autre, alors chaque sélection est mémorisée séparément (jamais substituée par l'autre type d'unité).</t>
         </is>
       </c>
+      <c r="O125" s="2" t="n"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -15013,7 +15337,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15039,6 +15362,7 @@
           <t>Étant donné une sélection de captages, quand j'ajoute une sélection de BVAEP, alors les deux coexistent et restent affichées distinctement dans les composants dédiés.</t>
         </is>
       </c>
+      <c r="O126" s="2" t="n"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -15081,7 +15405,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15107,6 +15430,7 @@
           <t>Étant donné la bascule d'échelle, quand je reviens aux captages, alors la sélection de captages d'origine est restituée à l'identique.</t>
         </is>
       </c>
+      <c r="O127" s="2" t="n"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -15149,7 +15473,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15175,6 +15498,7 @@
           <t>Étant donné une liste d'unités, quand je choisis « Tri par nom », alors la liste est triée par ordre alphabétique (avec sens ascendant/descendant), sans modifier la sélection.</t>
         </is>
       </c>
+      <c r="O128" s="2" t="n"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -15217,7 +15541,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15243,6 +15566,7 @@
           <t>Étant donné une liste, quand je choisis « Tri par distance », alors la liste ordonne les unités des plus proches aux plus éloignées par rapport à la référence définie (position de recherche ou point central courant).</t>
         </is>
       </c>
+      <c r="O129" s="2" t="n"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -15285,7 +15609,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15311,6 +15634,7 @@
           <t>Étant donné un tri en cours, quand je change de mode, alors l'autre mode s'applique immédiatement.</t>
         </is>
       </c>
+      <c r="O130" s="2" t="n"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -15353,7 +15677,6 @@
           <t>Cartographie &amp; exploration &gt; Sélecteur de captages / BV</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -15379,6 +15702,7 @@
           <t>Étant donné un tri appliqué, quand j'ajoute ou je retire des unités, alors l'ordre est recalculé en conservant le mode choisi.</t>
         </is>
       </c>
+      <c r="O131" s="2" t="n"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -15451,6 +15775,7 @@
           <t>Étant donné un bassin versant et le référentiel communal, quand le calcul d'intersection est exécuté, alors sont identifiées les communes dont la surface intersectée avec le bassin versant atteint au moins 20 % de la surface du bassin.</t>
         </is>
       </c>
+      <c r="O132" s="2" t="n"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -15523,6 +15848,7 @@
           <t>Étant donné une commune dont le taux d'intersection est inférieur au seuil de 20 %, quand le calcul est exécuté, alors elle n'est pas retenue pour la facette « Commune ».</t>
         </is>
       </c>
+      <c r="O133" s="2" t="n"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -15595,6 +15921,7 @@
           <t>Étant donné un bassin versant mis à jour (US3.1), quand le calcul est relancé, alors la liste des communes de la facette reflète les relations à jour du référentiel.</t>
         </is>
       </c>
+      <c r="O134" s="2" t="n"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -15667,6 +15994,7 @@
           <t>Étant donné la facette « Commune » de la recherche (US6.10), quand elle est alimentée par ce calcul, alors elle ne présente que les communes validées par la règle (≥ 20 %), cohérentes avec la sélection courante des bassins versants.</t>
         </is>
       </c>
+      <c r="O135" s="2" t="n"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -15739,6 +16067,7 @@
           <t>Étant donné un calcul exécuté, quand le seuil ou le référentiel ont été modifiés, alors le recalcul est rejouable et trace les paramètres utilisés (seuil, version du référentiel), sans saisie manuelle.</t>
         </is>
       </c>
+      <c r="O136" s="2" t="n"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -15811,6 +16140,7 @@
           <t>Étant donné des captages appartenant à des BVAEP, quand je demande la mise en évidence du croisement, alors les liens captage → bassin versant sont explicites et lisibles sur la carte.</t>
         </is>
       </c>
+      <c r="O137" s="2" t="n"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -15883,6 +16213,7 @@
           <t>Étant donné la mise en évidence active, quand je survole un captage, alors le ou les bassins versants associés se mettent en avant (et inversement).</t>
         </is>
       </c>
+      <c r="O138" s="2" t="n"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -15955,6 +16286,7 @@
           <t>Étant donné le croisement affiché, quand un captage est hors bassin, alors il est distinguable et signalé comme « hors bassin » (pas de lien forcé).</t>
         </is>
       </c>
+      <c r="O139" s="2" t="n"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -16027,6 +16359,7 @@
           <t>Étant donné un référentiel mis à jour (US3.1 / US3.2), quand la carte est rafraîchie, alors le croisement restitué utilise les relations à jour.</t>
         </is>
       </c>
+      <c r="O140" s="2" t="n"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -16069,7 +16402,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr"/>
       <c r="J141" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16095,6 +16427,7 @@
           <t>Étant donné la carte, quand j'ouvre le sélecteur de fond posé sur la carte, alors les trois choix « Cartographie », « Satellite », « Terrain » sont proposés.</t>
         </is>
       </c>
+      <c r="O141" s="2" t="n"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -16137,7 +16470,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I142" t="inlineStr"/>
       <c r="J142" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16163,6 +16495,7 @@
           <t>Étant donné le choix d'un fond, quand je le valide, alors la carte bascule immédiatement sur ce fond en conservant couches, indicateur et emprise courants.</t>
         </is>
       </c>
+      <c r="O142" s="2" t="n"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -16205,7 +16538,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr"/>
       <c r="J143" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16231,6 +16563,7 @@
           <t>Étant donné un fond sans couverture (ex. satellite hors zone), quand il est sélectionné, alors un fond de substitution est affiché sans erreur visible.</t>
         </is>
       </c>
+      <c r="O143" s="2" t="n"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -16273,7 +16606,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr"/>
       <c r="J144" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16299,6 +16631,7 @@
           <t>Étant donné le choix du fond, quand ma préférence est mémorisée, alors elle est ré-appliquée lors des prochaines sessions.</t>
         </is>
       </c>
+      <c r="O144" s="2" t="n"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -16341,7 +16674,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
       <c r="J145" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16367,6 +16699,7 @@
           <t>Étant donné le volet gauche avec la section « Couches », quand la vue est ouverte, alors chaque couche est listée (BVAEP, captages, PPE – périmètres de protection, zones à risque) avec son état de visibilité.</t>
         </is>
       </c>
+      <c r="O145" s="2" t="n"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -16409,7 +16742,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
       <c r="J146" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16435,6 +16767,7 @@
           <t>Étant donné un basculement de couche, quand je l'affiche, alors elle apparaît immédiatement ; quand je la masque, elle disparaît sans impact sur les autres couches.</t>
         </is>
       </c>
+      <c r="O146" s="2" t="n"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -16477,7 +16810,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I147" t="inlineStr"/>
       <c r="J147" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16503,6 +16835,7 @@
           <t>Étant donné un indicateur porté par la couche BVAEP, quand la couche est masquée, alors le rendu de l'indicateur est mis en évidence (message proposant sa réactivation) au lieu d'un affichage silencieusement vide.</t>
         </is>
       </c>
+      <c r="O147" s="2" t="n"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -16545,7 +16878,6 @@
           <t>Cartographie &amp; exploration &gt; Cartographie</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr"/>
       <c r="J148" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16571,6 +16903,7 @@
           <t>Étant donné plusieurs couches actives, quand elles se superposent, alors l'ordre de rendu est stable et la lisibilité est conservée.</t>
         </is>
       </c>
+      <c r="O148" s="2" t="n"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -16613,7 +16946,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16639,6 +16971,7 @@
           <t>Étant donné le menu déroulant des indicateurs, quand je le déploie, alors la liste est hiérarchisée Famille → Thème → Groupe.</t>
         </is>
       </c>
+      <c r="O149" s="2" t="n"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -16681,7 +17014,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16707,6 +17039,7 @@
           <t>Étant donné la hiérarchie, quand je navigue niveau par niveau, alors la recherche restreint la liste aux choix descendants du niveau actif.</t>
         </is>
       </c>
+      <c r="O150" s="2" t="n"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -16749,7 +17082,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16775,6 +17107,7 @@
           <t>Étant donné un texte saisi, quand il correspond à des indicateurs, alors la liste filtrée les présente avec leur libellé, sans ambiguïté.</t>
         </is>
       </c>
+      <c r="O151" s="2" t="n"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -16817,7 +17150,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16843,6 +17175,7 @@
           <t>Étant donné l'indicateur choisi, quand je le valide, alors le catalogue indicateurs et la carte se mettent à jour.</t>
         </is>
       </c>
+      <c r="O152" s="2" t="n"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -16885,7 +17218,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16911,6 +17243,7 @@
           <t>Étant donné la vignette d'un indicateur, quand je la sélectionne pour les métadonnées, alors la fiche métadonnées s'ouvre.</t>
         </is>
       </c>
+      <c r="O153" s="2" t="n"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -16953,7 +17286,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -16979,6 +17311,7 @@
           <t>Étant donné la fiche métadonnées affichée, alors elle contient la définition, l'unité, la période, les sources et le lignage des données mobilisées (catalogue).</t>
         </is>
       </c>
+      <c r="O154" s="2" t="n"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -17021,7 +17354,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17047,6 +17379,7 @@
           <t>Étant donné la règle d'accès, quand je tente d'ouvrir les métadonnées depuis un graphique, alors l'entrée n'est pas activée (accès uniquement depuis la vignette).</t>
         </is>
       </c>
+      <c r="O155" s="2" t="n"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -17089,7 +17422,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17115,6 +17447,7 @@
           <t>Étant donné une fiche métadonnées d'indicateur, quand elle est consultée, alors elle est cohérente avec le catalogue de référence même si l'indicateur n'est pas encore calculé.</t>
         </is>
       </c>
+      <c r="O156" s="2" t="n"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -17157,7 +17490,6 @@
           <t>Cartographie &amp; exploration &gt; Visualisation &amp; dataviz</t>
         </is>
       </c>
-      <c r="I157" t="inlineStr"/>
       <c r="J157" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17183,6 +17515,7 @@
           <t>Étant donné un graphique d'indicateur, quand il est consulté, alors les bascules « Répartition », « Temporel », « Changements » et « Carte » sont disponibles.</t>
         </is>
       </c>
+      <c r="O157" s="2" t="n"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -17225,7 +17558,6 @@
           <t>Cartographie &amp; exploration &gt; Visualisation &amp; dataviz</t>
         </is>
       </c>
-      <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17251,6 +17583,7 @@
           <t>Étant donné un indicateur sans historique, quand la vue « Temporel » serait demandée, alors elle est désactivée (grisée) avec le commentaire « données non historisées ».</t>
         </is>
       </c>
+      <c r="O158" s="2" t="n"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -17293,7 +17626,6 @@
           <t>Cartographie &amp; exploration &gt; Visualisation &amp; dataviz</t>
         </is>
       </c>
-      <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17319,6 +17651,7 @@
           <t>Étant donné une vue active, quand je bascule entre les vues, alors l'indicateur, la sélection et la période courants sont transmis à la nouvelle vue.</t>
         </is>
       </c>
+      <c r="O159" s="2" t="n"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -17361,7 +17694,6 @@
           <t>Cartographie &amp; exploration &gt; Visualisation &amp; dataviz</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17387,6 +17719,7 @@
           <t>Étant donné la vue « Changements » demandée, quand les données sont insuffisantes, alors un état « données insuffisantes » est affiché au lieu d'un faux résultat.</t>
         </is>
       </c>
+      <c r="O160" s="2" t="n"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -17429,7 +17762,6 @@
           <t>Cartographie &amp; exploration &gt; Visualisation &amp; dataviz</t>
         </is>
       </c>
-      <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17455,6 +17787,7 @@
           <t>Étant donné un indicateur, quand la vue « Carte » (maille H3) est affichée, alors elle est cohérente avec la carte principale (classes et palettes identiques).</t>
         </is>
       </c>
+      <c r="O161" s="2" t="n"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -17497,7 +17830,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17523,6 +17855,7 @@
           <t>Étant donné le catalogue d'indicateurs complet, quand je l'ouvre, alors la liste complète (38 indicateurs) s'affiche, regroupée par Famille → Thème → Groupe avec compteurs.</t>
         </is>
       </c>
+      <c r="O162" s="2" t="n"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -17565,7 +17898,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I163" t="inlineStr"/>
       <c r="J163" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17591,6 +17923,7 @@
           <t>Étant donné un regroupement, quand une famille/thème est sans indicateur visible, alors elle est affichée vide ou masquée selon une règle cohérente, jamais tronquée arbitrairement.</t>
         </is>
       </c>
+      <c r="O163" s="2" t="n"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -17633,7 +17966,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I164" t="inlineStr"/>
       <c r="J164" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17659,6 +17991,7 @@
           <t>Étant donné le catalogue des indicateurs, quand je recherche par libellé, alors le résultat reste hiérarchisé et identifiable.</t>
         </is>
       </c>
+      <c r="O164" s="2" t="n"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -17701,7 +18034,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I165" t="inlineStr"/>
       <c r="J165" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17727,6 +18059,7 @@
           <t>Étant donné les droits du profil, quand un indicateur n'est pas autorisé, alors il est absent de la liste pour ce profil, sans message d'erreur.</t>
         </is>
       </c>
+      <c r="O165" s="2" t="n"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -17769,7 +18102,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17795,6 +18127,7 @@
           <t>Étant donné le volet droit des indicateurs, quand il est affiché, alors les onglets (tabs) par famille, les pastilles (pills) par thème et le menu déroulant par groupe sont disponibles.</t>
         </is>
       </c>
+      <c r="O166" s="2" t="n"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -17837,7 +18170,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I167" t="inlineStr"/>
       <c r="J167" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17863,6 +18195,7 @@
           <t>Étant donné une famille sélectionnée, quand des pastilles (pills) sont choisies, alors la liste des groupes d'indicateurs est pré-sélectionnée en conséquence.</t>
         </is>
       </c>
+      <c r="O167" s="2" t="n"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -17905,7 +18238,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I168" t="inlineStr"/>
       <c r="J168" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17931,6 +18263,7 @@
           <t>Étant donné une pré-sélection appliquée, quand le volet droit est rendu, alors l'indicateur proposé est en cohérence avec les thèmes et le groupe sélectionnés.</t>
         </is>
       </c>
+      <c r="O168" s="2" t="n"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -17973,7 +18306,6 @@
           <t>Cartographie &amp; exploration &gt; Catalogue d'indicateurs</t>
         </is>
       </c>
-      <c r="I169" t="inlineStr"/>
       <c r="J169" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -17999,6 +18331,7 @@
           <t>Étant donné une navigation entre familles, quand je change de tab, alors la pré-sélection de la nouvelle famille s'applique sans confusion avec la précédente.</t>
         </is>
       </c>
+      <c r="O169" s="2" t="n"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -18041,7 +18374,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I170" t="inlineStr"/>
       <c r="J170" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18067,6 +18399,7 @@
           <t>Étant donné une sélection courante (captages / BVAEP, indicateurs, facettes), quand je lance l'export CSV, alors un fichier CSV est téléchargé couvrant l'ensemble du périmètre sélectionné (filtres inclus).</t>
         </is>
       </c>
+      <c r="O170" s="2" t="n"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -18109,7 +18442,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I171" t="inlineStr"/>
       <c r="J171" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18135,6 +18467,7 @@
           <t>Étant donné le fichier téléchargé, quand je l'ouvre dans un tableur, alors il est encodé UTF-8 (BOM), avec séparateur cohérent, ligne d'entête et ligne par unité/valeur.</t>
         </is>
       </c>
+      <c r="O171" s="2" t="n"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -18177,7 +18510,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18203,6 +18535,7 @@
           <t>Étant donné les colonnes de l'export, quand le fichier est produit, alors elles sont nommées et documentées (identifiant, nom, échelle, période, valeur, unité) et cohérentes avec la vue affichée.</t>
         </is>
       </c>
+      <c r="O172" s="2" t="n"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -18245,7 +18578,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18271,6 +18603,7 @@
           <t>Étant donné une valeur absente, quand le fichier est rempli, alors la cellule est vide avec un code « NA » documenté (jamais un zéro à la place d'une donnée inconnue).</t>
         </is>
       </c>
+      <c r="O173" s="2" t="n"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -18313,7 +18646,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18339,6 +18671,7 @@
           <t>Étant donné un volume important, quand l'export est demandé, alors le résultat est complet (pagination interne, sans perte silencieuse) et la préparation est signalée si nécessaire.</t>
         </is>
       </c>
+      <c r="O174" s="2" t="n"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -18381,7 +18714,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18407,6 +18739,7 @@
           <t>Étant donné une « vue simple » en consultation, quand j'en demande l'export, alors je reçois un fichier consolidé et simple de la vue courante : sélection, indicateurs, période et facettes appliquées.</t>
         </is>
       </c>
+      <c r="O175" s="2" t="n"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -18449,7 +18782,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I176" t="inlineStr"/>
       <c r="J176" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18475,6 +18807,7 @@
           <t>Étant donné l'export de vue simple, quand il est produit, alors son contenu correspond à la vue affichée à l'écran au moment de l'export (ni plus, ni moins).</t>
         </is>
       </c>
+      <c r="O176" s="2" t="n"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -18517,7 +18850,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I177" t="inlineStr"/>
       <c r="J177" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18543,6 +18875,7 @@
           <t>Étant donné la vue simple, quand l'export est déclenché, alors une seule action suffit, sans paramétrage avancé (adapté aux utilisateurs non techniques).</t>
         </is>
       </c>
+      <c r="O177" s="2" t="n"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -18585,7 +18918,6 @@
           <t>Export &amp; diffusion</t>
         </is>
       </c>
-      <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>Restitution – Diffusion</t>
@@ -18611,6 +18943,7 @@
           <t>Étant donné l'export de vue simple, quand le fichier est ouvert, alors les métadonnées d'en-tête (nom de la vue, date d'export, source « HydroScope ») précisent le périmètre diffusé.</t>
         </is>
       </c>
+      <c r="O178" s="2" t="n"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -18653,7 +18986,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -18679,6 +19011,7 @@
           <t>Étant donné des identifiants valides, quand je me connecte, alors l'authentification réussit et je suis redirigé vers la vue de mon profil, sans mot de passe affiché ni stocké en clair.</t>
         </is>
       </c>
+      <c r="O179" s="2" t="n"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -18721,7 +19054,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I180" t="inlineStr"/>
       <c r="J180" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -18747,6 +19079,7 @@
           <t>Étant donné des identifiants invalides, quand je tente une connexion, alors un message d'échec générique est affiché et l'incident (échec) est tracé côté logs.</t>
         </is>
       </c>
+      <c r="O180" s="2" t="n"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -18789,7 +19122,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -18815,6 +19147,7 @@
           <t>Étant donné une session authentifiée, quand celle-ci expire (inactivité définie), alors l'utilisateur est déconnecté proprement et redirigé vers le formulaire de connexion.</t>
         </is>
       </c>
+      <c r="O181" s="2" t="n"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -18857,7 +19190,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -18883,6 +19215,7 @@
           <t>Étant donné une fonctionnalité protégée, quand un utilisateur non authentifié tente d'y accéder, alors une redirection vers l'authentification est effectuée avant de servir la ressource.</t>
         </is>
       </c>
+      <c r="O182" s="2" t="n"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -18925,7 +19258,6 @@
           <t>Administration &amp; profils</t>
         </is>
       </c>
-      <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -18951,6 +19283,7 @@
           <t>Étant donné la conformité RGPD (cookies / stockage local), quand une session est ouverte, alors aucun mot de passe ni donnée personnelle sensible n'est stocké côté navigateur.</t>
         </is>
       </c>
+      <c r="O183" s="2" t="n"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -19023,6 +19356,7 @@
           <t>Étant donné les rôles définis par la plateforme (administrateur plateforme, administrateur expert data, expert métier eau potable, décideur, intéressé public), quand un compte est créé ou modifié, alors un rôle simple lui est attribué parmi cette liste normative.</t>
         </is>
       </c>
+      <c r="O184" s="2" t="n"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -19095,6 +19429,7 @@
           <t>Étant donné un utilisateur connecté, quand il utilise la plateforme, alors seules les fonctionnalités autorisées par son rôle sont visibles et actives.</t>
         </is>
       </c>
+      <c r="O185" s="2" t="n"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -19167,6 +19502,7 @@
           <t>Étant donné un utilisateur sans droit, quand il tente d'accéder à une fonctionnalité ou URL directe, alors l'accès est bloqué (aucun contournement par autorisation via adresse directe).</t>
         </is>
       </c>
+      <c r="O186" s="2" t="n"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -19239,6 +19575,7 @@
           <t>Étant donné le changement de rôle d'un compte, quand il est enregistré, alors les nouveaux droits sont appliqués à la connexion suivante, sans privilège résiduel sur la session antérieure.</t>
         </is>
       </c>
+      <c r="O187" s="2" t="n"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -19281,7 +19618,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -19307,6 +19643,7 @@
           <t>Étant donné un import (fichier ou source externe) réalisé, quand il se termine, alors une entrée de journal est créée : type d'import, source, périmètre, nombre de lignes, statut (réussi / partiel / échoué) et horaire (dates/heures).</t>
         </is>
       </c>
+      <c r="O188" s="2" t="n"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -19349,7 +19686,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I189" t="inlineStr"/>
       <c r="J189" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -19375,6 +19711,7 @@
           <t>Étant donné un import partiel ou échoué, quand l'entrée est consultée, alors les détails des erreurs (lignes rejetées, motif) sont accessibles pour la correction.</t>
         </is>
       </c>
+      <c r="O189" s="2" t="n"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -19417,7 +19754,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I190" t="inlineStr"/>
       <c r="J190" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -19443,6 +19779,7 @@
           <t>Étant donné le journal des imports, quand je le consulte, alors la recherche par période, source et statut est possible, et le contenu est immuable (aucune suppression).</t>
         </is>
       </c>
+      <c r="O190" s="2" t="n"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -19485,7 +19822,6 @@
           <t>Suivi qualité &amp; traçabilité</t>
         </is>
       </c>
-      <c r="I191" t="inlineStr"/>
       <c r="J191" t="inlineStr">
         <is>
           <t>Gouvernance</t>
@@ -19511,6 +19847,7 @@
           <t>Étant donné un import suivi, quand il est enregistré, alors l'événement est visible dans le journal dans un délai conforme aux engagements contractuels, indépendamment du statut ultérieur des données.</t>
         </is>
       </c>
+      <c r="O191" s="2" t="n"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -19583,6 +19920,7 @@
           <t>Étant donné un calcul (indicateur simple, agrégation bassin versant, agrégation temporelle) exécuté, quand il est journalisé, alors le journal enregistre : identifiant de l'exécution, version de l'indicateur, données d'entrée, paramètres, date et statut.</t>
         </is>
       </c>
+      <c r="O192" s="2" t="n"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -19655,6 +19993,7 @@
           <t>Étant donné un recalcul, quand il est déclenché, alors une nouvelle entrée de journal est créée (l'entrée précédente n'est pas écrasée), permettant la reconstitution.</t>
         </is>
       </c>
+      <c r="O193" s="2" t="n"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -19727,6 +20066,7 @@
           <t>Étant donné le journal des calculs, quand je le consulte, alors il permet de relier chaque résultat à la définition d'indicateur et aux paramètres utilisés.</t>
         </is>
       </c>
+      <c r="O194" s="2" t="n"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -19799,6 +20139,7 @@
           <t>Étant donné l'échec d'un calcul, quand il est journalisé, alors le motif est explicité, accessible à l'administrateur pour permettre la correction.</t>
         </is>
       </c>
+      <c r="O195" s="2" t="n"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -19841,7 +20182,6 @@
           <t>Suivi &amp; veille</t>
         </is>
       </c>
-      <c r="I196" t="inlineStr"/>
       <c r="J196" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -19867,6 +20207,7 @@
           <t>Étant donné un indicateur historisé, quand l'analyse est déclenchée, alors une tendance (orientation : hausse, baisse, stable) est affichée avec sa période de référence.</t>
         </is>
       </c>
+      <c r="O196" s="2" t="n"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -19909,7 +20250,6 @@
           <t>Suivi &amp; veille</t>
         </is>
       </c>
-      <c r="I197" t="inlineStr"/>
       <c r="J197" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -19935,6 +20275,7 @@
           <t>Étant donné la tendance calculée, quand je la consulte, alors l'intensité (delta ou seuil de variation) présentée est fondée sur une règle explicite et reproductible.</t>
         </is>
       </c>
+      <c r="O197" s="2" t="n"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -19977,7 +20318,6 @@
           <t>Suivi &amp; veille</t>
         </is>
       </c>
-      <c r="I198" t="inlineStr"/>
       <c r="J198" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -20003,6 +20343,7 @@
           <t>Étant donné une tendance détectée, quand je survole l'élément, alors les valeurs montrant l'évolution de la période sont détaillées.</t>
         </is>
       </c>
+      <c r="O198" s="2" t="n"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -20045,7 +20386,6 @@
           <t>Suivi &amp; veille</t>
         </is>
       </c>
-      <c r="I199" t="inlineStr"/>
       <c r="J199" t="inlineStr">
         <is>
           <t>Exploitation</t>
@@ -20071,6 +20411,7 @@
           <t>Étant donné une série trop courte pour une tendance significative, quand elle est demandée, alors l'état « historique insuffisant » est affiché au lieu d'un résultat indicatif.</t>
         </is>
       </c>
+      <c r="O199" s="2" t="n"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -20143,6 +20484,7 @@
           <t>Étant donné une règle de détection configurée (seuils US7.1, tendances US7.3), quand la valeur d'un indicateur sur un captage ou BVAEP franchit le critère de changement significatif, alors une alerte au changement est levée, datée et qualifiée. -</t>
         </is>
       </c>
+      <c r="O200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -20215,6 +20557,7 @@
           <t>Étant donné une alerte levée, quand je consulte son détail, alors la règle déclencheuse (indicateur, delta, période comparée, seuil) est exposée de façon explicite et reproductible. -</t>
         </is>
       </c>
+      <c r="O201" s="2" t="n"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -20287,6 +20630,7 @@
           <t>Étant donné un captage/BVAEP avec une alerte active, quand je consulte sa fiche ou sa vue, alors les indicateurs ayant évolué sont mis en évidence (badge/teinte), sans aucune notification poussée (consultation seule). -</t>
         </is>
       </c>
+      <c r="O202" s="2" t="n"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -20359,6 +20703,7 @@
           <t>Étant donné une vue présentant plusieurs signalements, quand ils coexistent, alors l'alerte au changement est distinguée du dépassement de seuil (US7.1) et de la tendance (US7.3). -</t>
         </is>
       </c>
+      <c r="O203" s="2" t="n"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -20431,6 +20776,7 @@
           <t>Étant donné une alerte active, quand la valeur revient sous le critère ou la période de référence change, alors l'alerte est levée ou marquée « en résolution », sans message résiduel trompeur. -</t>
         </is>
       </c>
+      <c r="O204" s="2" t="n"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -20503,6 +20849,7 @@
           <t>Étant donné le suivi d'un captage/BVAEP, quand je consulte l'historique, alors les alertes passées restent consultables (date, règle, état) sans être écrasées. -</t>
         </is>
       </c>
+      <c r="O205" s="2" t="n"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -20575,6 +20922,7 @@
           <t>Étant donné une série trop courte ou non historisée, quand une alerte serait candidate, alors l'état « historique insuffisant » est affiché et aucune alerte due n'est levée. -</t>
         </is>
       </c>
+      <c r="O206" s="2" t="n"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -20647,8 +20995,10 @@
           <t>Étant donné un profil habilité, quand une alerte est active ou configurée, alors la lecture respecte les droits (RBAC) et la configuration reste tracée (utilisateur, date).</t>
         </is>
       </c>
+      <c r="O207" s="2" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A1:N207"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Implement caching server for HydroScope with FastAPI and SQLite
- Added database management with SQLite for caching sources and features.
- Created API endpoints for listing sources, fetching features, and refreshing cache.
- Implemented asynchronous data synchronization from ArcGIS services.
- Developed frontend context and components for managing and displaying referential data.
- Configured Docker for containerized deployment of the caching server.
- Added health check and environment variable support for TTL configuration.
</commit_message>
<xml_diff>
--- a/cahier des charges/backlog.xlsx
+++ b/cahier des charges/backlog.xlsx
@@ -3393,7 +3393,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3466,8 +3466,10 @@
         <v>22</v>
       </c>
       <c r="L2" s="1" t="n">
-        <f aca="false">SUMIF('Besoins testables'!$D:$D,$A2,'Besoins testables'!$O:$O)</f>
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="M2" s="0" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4323,7 +4325,10 @@
       <c r="K26" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="L26" s="1"/>
+      <c r="L26" s="1" t="n">
+        <f aca="false">SUMIF('Besoins testables'!$D:$D,$A26,'Besoins testables'!$O:$O)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
@@ -6829,7 +6834,7 @@
       </c>
       <c r="L96" s="1"/>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
         <v>345</v>
       </c>

</xml_diff>

<commit_message>
CDC/MD: soldes C (libellés/3W/profils, EPIC1-4) + P11 — Proposé par Marjolaine David (backlog-v1.1-MD-commentaires.xlsx) — décision: intégré (C2-C3,C6,C11-C12,C17,C19,C22-C24,C26,C28-C29,C31,C33-C34,C36 + P11 alertes ; C5,C16,C24-conforme,C40 déjà conformes ; C35 conservée motivée ; C37-C39 admin confirmé 3.2)
</commit_message>
<xml_diff>
--- a/cahier des charges/backlog.xlsx
+++ b/cahier des charges/backlog.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Planifier des imports simples</t>
+          <t>Planifier des intégrations simples</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux planifier des imports simples afin que les données soient actualisées automatiquement.</t>
+          <t>En tant qu'administrateur expert data, je veux planifier des intégrations simples afin que les données soient actualisées automatiquement.</t>
         </is>
       </c>
       <c r="L4" s="1">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Alimenter automatiquement le catalogue lors des imports</t>
+          <t>Alimenter automatiquement le catalogue lors des intégrations de données</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux alimenter automatiquement le catalogue lors des imports afin d'éviter les saisies manuelles.</t>
+          <t>En tant qu'administrateur expert data, je veux alimenter automatiquement le catalogue lors des intégrations de données afin d'éviter les saisies manuelles.</t>
         </is>
       </c>
       <c r="L18" s="1">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="K27" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux calculer un taux de complétude afin de mesurer la couverture des données.</t>
+          <t>En tant qu'administrateur expert data, je veux calculer un taux de complétude afin de mesurer la couverture des données sur le territoire de la Nouvelle-Calédonie.</t>
         </is>
       </c>
       <c r="L27" s="1">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>Définir un indicateur</t>
+          <t>Décrire un indicateur au référentiel</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="K35" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux définir un indicateur afin de le rendre calculable et affichable.</t>
+          <t>En tant qu'administrateur expert data, je veux décrire un indicateur au référentiel (méthode de calcul) afin de le rendre calculable (précalcul, sans création via le front) et affichable.</t>
         </is>
       </c>
       <c r="L35" s="1">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="K42" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux filtrer les données afin de restreindre le calcul aux valeurs pertinentes.</t>
+          <t>En tant qu'administrateur expert data, je veux filtrer les données en amont des calculs (traitements codés en dur, sans filtre via le front) afin de restreindre le calcul aux valeurs pertinentes.</t>
         </is>
       </c>
       <c r="L42" s="1">
@@ -2921,7 +2921,7 @@
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>Définir des pondérations</t>
+          <t>Choisir un jeu de pondérations de référence</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'expert métier eau potable, je veux définir les pondérations de l'analyse multicritère afin d'évaluer le risque réel de dégradation de la ressource.</t>
+          <t>En tant qu'expert métier eau potable, je veux choisir un jeu de pondérations de référence (avec sa fiche méthodo) pour l'analyse multicritère afin d'évaluer le risque réel de dégradation de la ressource.</t>
         </is>
       </c>
       <c r="L46" s="1" t="n"/>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="K47" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'expert métier eau potable, je veux tester des scénarios de pondération afin d'analyser l'impact des différents facteurs sur le classement de criticité.</t>
+          <t>En tant qu'expert métier eau potable, je veux tester des scénarios de pondération afin d'analyser l'impact des différents facteurs sur le classement multicritère.</t>
         </is>
       </c>
       <c r="L47" s="1" t="n"/>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>Comparer scénarios</t>
+          <t>Comparer et partager des scénarios</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="K48" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'expert métier eau potable, je veux comparer les scénarios de l'analyse multicritère afin d'identifier la pondération la plus représentative du terrain.</t>
+          <t>En tant qu'expert métier eau potable, je veux comparer les scénarios de l'analyse multicritère afin d'identifier la pondération la plus représentative du terrain et de la partager (jeu de référence).</t>
         </is>
       </c>
       <c r="L48" s="1" t="n"/>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="K55" s="1" t="inlineStr">
         <is>
-          <t>En tant que décideur métier, je veux comparer des territoires afin d'arbitrer les investissements.</t>
+          <t>En tant que décideur métier, je veux comparer des territoires sur la base d'indicateurs agrégés afin d'arbitrer les investissements.</t>
         </is>
       </c>
       <c r="L55" s="1" t="n"/>
@@ -3637,12 +3637,12 @@
       </c>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Administrateur expert data</t>
+          <t>Expert métier eau potable</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux basculer l'échelle d'analyse entre captages et bassins versants afin de changer de niveau de lecture.</t>
+          <t>En tant qu'expert métier eau potable, je veux basculer l'échelle d'analyse entre captages et bassins versants afin de changer de niveau de lecture.</t>
         </is>
       </c>
       <c r="L58" s="1">
@@ -4085,12 +4085,12 @@
       </c>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Administrateur expert data</t>
+          <t>Expert métier eau potable</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux conserver indépendamment les sélections captages et bassins versants afin de ne pas les mélanger.</t>
+          <t>En tant qu'administrateur expert data, je veux conserver indépendamment les sélections captages, bassins versants et PPE afin de ne pas les mélanger.</t>
         </is>
       </c>
       <c r="L66" s="1">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux afficher ou masquer chaque couche afin de personnaliser ce qui est visible.</t>
+          <t>En tant qu'expert métier eau potable, je veux afficher ou masquer chaque couche afin de personnaliser ce qui est visible.</t>
         </is>
       </c>
       <c r="L71" s="1" t="inlineStr">
@@ -4488,12 +4488,12 @@
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>Administrateur expert data</t>
+          <t>Expert métier eau potable</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux consulter la fiche métadonnées d'un indicateur afin d'en vérifier la définition.</t>
+          <t>En tant qu'expert métier eau potable, je veux consulter la fiche métadonnées d'un indicateur afin d'en vérifier la définition.</t>
         </is>
       </c>
       <c r="L73" s="1">
@@ -4656,12 +4656,12 @@
       </c>
       <c r="J76" s="1" t="inlineStr">
         <is>
-          <t>Administrateur expert data</t>
+          <t>Expert métier eau potable</t>
         </is>
       </c>
       <c r="K76" s="1" t="inlineStr">
         <is>
-          <t>En tant qu'administrateur expert data, je veux présélectionner les indicateurs par famille afin d'orienter l'usage du volet droit.</t>
+          <t>En tant qu'expert métier / utilisateur, Je veux sélectionner individuellement les indicateurs à activer au sein de chaque famille thématique, Afin de personnaliser mon analyse et ne conserver que les métriques pertinentes pour mon étude.</t>
         </is>
       </c>
       <c r="L76" s="1">

</xml_diff>